<commit_message>
Add contact emails; drop per-professor research area labels
Contact: the Settings email field can now hold several addresses, shown
as a list on the Contact page and under the address on the home page.
Two addresses are filled in.

People: remove the Clinical / Translational chip from the principal
investigator cards and the area column from the People sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/glory-content.xlsx
+++ b/content/glory-content.xlsx
@@ -469,7 +469,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -477,7 +476,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -527,7 +525,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
@@ -570,7 +567,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
@@ -627,7 +623,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
@@ -646,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N400"/>
+  <dimension ref="A1:M400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -657,12 +652,12 @@
     <col width="34" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="46" customWidth="1" min="10" max="10"/>
+    <col width="46" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
-    <col width="60" customWidth="1" min="12" max="12"/>
-    <col width="70" customWidth="1" min="13" max="13"/>
-    <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="70" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -708,30 +703,25 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>affiliation</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>affiliation</t>
+          <t>research_interests</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>research_interests</t>
+          <t>education</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>education</t>
+          <t>career</t>
         </is>
       </c>
       <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>career</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>awards</t>
         </is>
@@ -780,30 +770,25 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>※ 담당 분야 (선택). PI 카드에 표시. 예) Clinical Research</t>
+          <t>※ 소속 (선택). 예) Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>※ 소속 (선택). 예) Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
+          <t>※ 연구 분야 (선택). 한 칸 안에서 Alt+Enter 로 줄을 바꾸면 항목이 나뉩니다</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>※ 연구 분야 (선택). 한 칸 안에서 Alt+Enter 로 줄을 바꾸면 항목이 나뉩니다</t>
+          <t>※ 학력 (선택). 한 줄에 한 항목 (Alt+Enter 로 줄바꿈)</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>※ 학력 (선택). 한 줄에 한 항목 (Alt+Enter 로 줄바꿈)</t>
+          <t>※ 경력 (선택). 한 줄에 한 항목 (Alt+Enter 로 줄바꿈)</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
-        <is>
-          <t>※ 경력 (선택). 한 줄에 한 항목 (Alt+Enter 로 줄바꿈)</t>
-        </is>
-      </c>
-      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>※ 수상 (선택). 한 줄에 한 항목 (Alt+Enter 로 줄바꿈)</t>
         </is>
@@ -840,29 +825,24 @@
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>Clinical Research</t>
+          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Radical surgery and hyperthermic intraperitoneal chemotherapy (HIPEC) for uterine and ovarian cancer
 Chemotherapy and novel agents for advanced and recurrent ovarian cancer
 Clinical trials to develop new treatments for uterine and ovarian cancer</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>2005  M.D., Hanyang University College of Medicine
 2010  M.S., Obstetrics and Gynecology, Seoul National University College of Medicine
 2015  Ph.D., Obstetrics and Gynecology, Seoul National University College of Medicine</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>2005–2006  Intern, Seoul National University Hospital
 2006–2010  Resident, Obstetrics and Gynecology, Seoul National University Hospital
@@ -878,7 +858,7 @@
 2020–present  Executive Committee, Asia-Pacific Gynecologic Oncology Trials Group (APGOT)</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="M3" s="4" t="inlineStr">
         <is>
           <t>2013  Commendation, Minister of Health and Welfare
 2016  LG Life Sciences Future Medical Scientist Award
@@ -920,29 +900,24 @@
       <c r="H4" s="4" t="n"/>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>Clinical Research</t>
+          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>Gynecologic cancer and sarcoma
 Minimally invasive and robotic surgery
 Chemotherapy, novel agents and clinical trials</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="K4" s="4" t="inlineStr">
         <is>
           <t>2007  B.S., Biochemistry, Yonsei University
 2012  M.D., Kyungpook National University School of Medicine
 2022  Ph.D., Obstetrics and Gynecology, Yonsei University College of Medicine</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>2012–2013  Intern, Severance Hospital
 2013–2017  Resident, Obstetrics and Gynecology, Severance Hospital
@@ -956,7 +931,7 @@
 Member, GCIG and APGOT</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="M4" s="4" t="inlineStr">
         <is>
           <t>2018  Best Oral Presentation, Korean Cancer Association
 2018  Best Oral Presentation, Korean Society of Obstetrics and Gynecology
@@ -996,29 +971,24 @@
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Translational Research</t>
+          <t>Department of Obstetrics and Gynecology, Soonchunhyang University Bucheon Hospital</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>Department of Obstetrics and Gynecology, Soonchunhyang University Bucheon Hospital</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>Tumor immunology and immunotherapy in gynecologic cancer
 Radical surgery for ovarian and uterine cancer
 Single-port laparoscopic and robotic surgery</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="K5" s="4" t="inlineStr">
         <is>
           <t>2010  M.D., Soonchunhyang University College of Medicine
 2013  M.S., Obstetrics and Gynecology, Soonchunhyang University College of Medicine
 2019  Ph.D., Immunology, Korea Advanced Institute of Science and Technology (KAIST)</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>2010–2011  Intern, Soonchunhyang University Bucheon Hospital
 2011–2015  Resident, Obstetrics and Gynecology, Soonchunhyang University Bucheon Hospital
@@ -1031,7 +1001,7 @@
 Member, American Association for Cancer Research and American Association of Immunologists</t>
         </is>
       </c>
-      <c r="N5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1064,15 +1034,10 @@
       <c r="H6" s="4" t="n"/>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Translational Research</t>
+          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Department of Obstetrics and Gynecology, Yonsei University College of Medicine</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>Precision and translational oncology in gynecologic cancers
 ctDNA/cfDNA, fragmentomics and minimal residual disease for early detection and longitudinal monitoring
@@ -1081,14 +1046,14 @@
 Precision trial design, including biomarker-guided treatment selection and escalation or de-escalation</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>2011  B.A., Economics and Biology, Columbia University
 2015  M.D., Yonsei University Graduate School of Medicine
 2023  Ph.D., Medicine, Yonsei University College of Medicine</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>2015–2016  Intern, Severance Hospital
 2016–2020  Resident, Obstetrics and Gynecology, Severance Hospital
@@ -1099,7 +1064,7 @@
 2026–present  Assistant Professor, Yonsei University College of Medicine</t>
         </is>
       </c>
-      <c r="N6" s="4" t="n"/>
+      <c r="M6" s="4" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1123,7 +1088,6 @@
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
       <c r="M7" s="4" t="n"/>
-      <c r="N7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1147,7 +1111,6 @@
       <c r="K8" s="4" t="n"/>
       <c r="L8" s="4" t="n"/>
       <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1171,7 +1134,6 @@
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
       <c r="M9" s="4" t="n"/>
-      <c r="N9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1195,7 +1157,6 @@
       <c r="K10" s="4" t="n"/>
       <c r="L10" s="4" t="n"/>
       <c r="M10" s="4" t="n"/>
-      <c r="N10" s="4" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1219,7 +1180,6 @@
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="n"/>
       <c r="M11" s="4" t="n"/>
-      <c r="N11" s="4" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1243,7 +1203,6 @@
       <c r="K12" s="4" t="n"/>
       <c r="L12" s="4" t="n"/>
       <c r="M12" s="4" t="n"/>
-      <c r="N12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1267,7 +1226,6 @@
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="n"/>
-      <c r="N13" s="4" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1291,7 +1249,6 @@
       <c r="K14" s="4" t="n"/>
       <c r="L14" s="4" t="n"/>
       <c r="M14" s="4" t="n"/>
-      <c r="N14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1315,7 +1272,6 @@
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="n"/>
       <c r="M15" s="4" t="n"/>
-      <c r="N15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1339,7 +1295,6 @@
       <c r="K16" s="4" t="n"/>
       <c r="L16" s="4" t="n"/>
       <c r="M16" s="4" t="n"/>
-      <c r="N16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1363,7 +1318,6 @@
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
       <c r="M17" s="4" t="n"/>
-      <c r="N17" s="4" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1387,7 +1341,6 @@
       <c r="K18" s="4" t="n"/>
       <c r="L18" s="4" t="n"/>
       <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1411,7 +1364,6 @@
       <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="n"/>
       <c r="M19" s="4" t="n"/>
-      <c r="N19" s="4" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1435,7 +1387,6 @@
       <c r="K20" s="4" t="n"/>
       <c r="L20" s="4" t="n"/>
       <c r="M20" s="4" t="n"/>
-      <c r="N20" s="4" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1459,7 +1410,6 @@
       <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="n"/>
       <c r="M21" s="4" t="n"/>
-      <c r="N21" s="4" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1483,7 +1433,6 @@
       <c r="K22" s="4" t="n"/>
       <c r="L22" s="4" t="n"/>
       <c r="M22" s="4" t="n"/>
-      <c r="N22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1507,7 +1456,6 @@
       <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="n"/>
       <c r="M23" s="4" t="n"/>
-      <c r="N23" s="4" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1535,7 +1483,6 @@
       <c r="K24" s="4" t="n"/>
       <c r="L24" s="4" t="n"/>
       <c r="M24" s="4" t="n"/>
-      <c r="N24" s="4" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1563,7 +1510,6 @@
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="n"/>
       <c r="M25" s="4" t="n"/>
-      <c r="N25" s="4" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1587,7 +1533,6 @@
       <c r="K26" s="4" t="n"/>
       <c r="L26" s="4" t="n"/>
       <c r="M26" s="4" t="n"/>
-      <c r="N26" s="4" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1611,7 +1556,6 @@
       <c r="K27" s="4" t="n"/>
       <c r="L27" s="4" t="n"/>
       <c r="M27" s="4" t="n"/>
-      <c r="N27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1635,7 +1579,6 @@
       <c r="K28" s="4" t="n"/>
       <c r="L28" s="4" t="n"/>
       <c r="M28" s="4" t="n"/>
-      <c r="N28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1659,7 +1602,6 @@
       <c r="K29" s="4" t="n"/>
       <c r="L29" s="4" t="n"/>
       <c r="M29" s="4" t="n"/>
-      <c r="N29" s="4" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="n"/>
@@ -1675,7 +1617,6 @@
       <c r="K30" s="4" t="n"/>
       <c r="L30" s="4" t="n"/>
       <c r="M30" s="4" t="n"/>
-      <c r="N30" s="4" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
@@ -1691,7 +1632,6 @@
       <c r="K31" s="4" t="n"/>
       <c r="L31" s="4" t="n"/>
       <c r="M31" s="4" t="n"/>
-      <c r="N31" s="4" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="n"/>
@@ -1707,7 +1647,6 @@
       <c r="K32" s="4" t="n"/>
       <c r="L32" s="4" t="n"/>
       <c r="M32" s="4" t="n"/>
-      <c r="N32" s="4" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
@@ -1723,7 +1662,6 @@
       <c r="K33" s="4" t="n"/>
       <c r="L33" s="4" t="n"/>
       <c r="M33" s="4" t="n"/>
-      <c r="N33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="n"/>
@@ -1739,7 +1677,6 @@
       <c r="K34" s="4" t="n"/>
       <c r="L34" s="4" t="n"/>
       <c r="M34" s="4" t="n"/>
-      <c r="N34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
@@ -1755,7 +1692,6 @@
       <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="n"/>
       <c r="M35" s="4" t="n"/>
-      <c r="N35" s="4" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="n"/>
@@ -1771,7 +1707,6 @@
       <c r="K36" s="4" t="n"/>
       <c r="L36" s="4" t="n"/>
       <c r="M36" s="4" t="n"/>
-      <c r="N36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
@@ -1787,7 +1722,6 @@
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="n"/>
       <c r="M37" s="4" t="n"/>
-      <c r="N37" s="4" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="n"/>
@@ -1803,7 +1737,6 @@
       <c r="K38" s="4" t="n"/>
       <c r="L38" s="4" t="n"/>
       <c r="M38" s="4" t="n"/>
-      <c r="N38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
@@ -1819,7 +1752,6 @@
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="n"/>
       <c r="M39" s="4" t="n"/>
-      <c r="N39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="n"/>
@@ -1835,7 +1767,6 @@
       <c r="K40" s="4" t="n"/>
       <c r="L40" s="4" t="n"/>
       <c r="M40" s="4" t="n"/>
-      <c r="N40" s="4" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
@@ -1851,7 +1782,6 @@
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="n"/>
       <c r="M41" s="4" t="n"/>
-      <c r="N41" s="4" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="n"/>
@@ -1867,7 +1797,6 @@
       <c r="K42" s="4" t="n"/>
       <c r="L42" s="4" t="n"/>
       <c r="M42" s="4" t="n"/>
-      <c r="N42" s="4" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
@@ -1883,7 +1812,6 @@
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="n"/>
       <c r="M43" s="4" t="n"/>
-      <c r="N43" s="4" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="n"/>
@@ -1899,7 +1827,6 @@
       <c r="K44" s="4" t="n"/>
       <c r="L44" s="4" t="n"/>
       <c r="M44" s="4" t="n"/>
-      <c r="N44" s="4" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
@@ -1915,7 +1842,6 @@
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="n"/>
       <c r="M45" s="4" t="n"/>
-      <c r="N45" s="4" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="n"/>
@@ -1931,7 +1857,6 @@
       <c r="K46" s="4" t="n"/>
       <c r="L46" s="4" t="n"/>
       <c r="M46" s="4" t="n"/>
-      <c r="N46" s="4" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
@@ -1947,7 +1872,6 @@
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="n"/>
       <c r="M47" s="4" t="n"/>
-      <c r="N47" s="4" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="n"/>
@@ -1963,7 +1887,6 @@
       <c r="K48" s="4" t="n"/>
       <c r="L48" s="4" t="n"/>
       <c r="M48" s="4" t="n"/>
-      <c r="N48" s="4" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
@@ -1979,7 +1902,6 @@
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="n"/>
       <c r="M49" s="4" t="n"/>
-      <c r="N49" s="4" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="n"/>
@@ -1995,7 +1917,6 @@
       <c r="K50" s="4" t="n"/>
       <c r="L50" s="4" t="n"/>
       <c r="M50" s="4" t="n"/>
-      <c r="N50" s="4" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
@@ -2011,7 +1932,6 @@
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="n"/>
       <c r="M51" s="4" t="n"/>
-      <c r="N51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="n"/>
@@ -2027,7 +1947,6 @@
       <c r="K52" s="4" t="n"/>
       <c r="L52" s="4" t="n"/>
       <c r="M52" s="4" t="n"/>
-      <c r="N52" s="4" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
@@ -2043,7 +1962,6 @@
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="n"/>
       <c r="M53" s="4" t="n"/>
-      <c r="N53" s="4" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="n"/>
@@ -2059,7 +1977,6 @@
       <c r="K54" s="4" t="n"/>
       <c r="L54" s="4" t="n"/>
       <c r="M54" s="4" t="n"/>
-      <c r="N54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="n"/>
@@ -2075,7 +1992,6 @@
       <c r="K55" s="4" t="n"/>
       <c r="L55" s="4" t="n"/>
       <c r="M55" s="4" t="n"/>
-      <c r="N55" s="4" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="n"/>
@@ -2091,7 +2007,6 @@
       <c r="K56" s="4" t="n"/>
       <c r="L56" s="4" t="n"/>
       <c r="M56" s="4" t="n"/>
-      <c r="N56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="n"/>
@@ -2107,7 +2022,6 @@
       <c r="K57" s="4" t="n"/>
       <c r="L57" s="4" t="n"/>
       <c r="M57" s="4" t="n"/>
-      <c r="N57" s="4" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="n"/>
@@ -2123,7 +2037,6 @@
       <c r="K58" s="4" t="n"/>
       <c r="L58" s="4" t="n"/>
       <c r="M58" s="4" t="n"/>
-      <c r="N58" s="4" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="n"/>
@@ -2139,7 +2052,6 @@
       <c r="K59" s="4" t="n"/>
       <c r="L59" s="4" t="n"/>
       <c r="M59" s="4" t="n"/>
-      <c r="N59" s="4" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="n"/>
@@ -2155,7 +2067,6 @@
       <c r="K60" s="4" t="n"/>
       <c r="L60" s="4" t="n"/>
       <c r="M60" s="4" t="n"/>
-      <c r="N60" s="4" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="n"/>
@@ -2171,7 +2082,6 @@
       <c r="K61" s="4" t="n"/>
       <c r="L61" s="4" t="n"/>
       <c r="M61" s="4" t="n"/>
-      <c r="N61" s="4" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="n"/>
@@ -2187,7 +2097,6 @@
       <c r="K62" s="4" t="n"/>
       <c r="L62" s="4" t="n"/>
       <c r="M62" s="4" t="n"/>
-      <c r="N62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="n"/>
@@ -2203,7 +2112,6 @@
       <c r="K63" s="4" t="n"/>
       <c r="L63" s="4" t="n"/>
       <c r="M63" s="4" t="n"/>
-      <c r="N63" s="4" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="4" t="n"/>
@@ -2219,7 +2127,6 @@
       <c r="K64" s="4" t="n"/>
       <c r="L64" s="4" t="n"/>
       <c r="M64" s="4" t="n"/>
-      <c r="N64" s="4" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="4" t="n"/>
@@ -2235,7 +2142,6 @@
       <c r="K65" s="4" t="n"/>
       <c r="L65" s="4" t="n"/>
       <c r="M65" s="4" t="n"/>
-      <c r="N65" s="4" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="n"/>
@@ -2251,7 +2157,6 @@
       <c r="K66" s="4" t="n"/>
       <c r="L66" s="4" t="n"/>
       <c r="M66" s="4" t="n"/>
-      <c r="N66" s="4" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="n"/>
@@ -2267,7 +2172,6 @@
       <c r="K67" s="4" t="n"/>
       <c r="L67" s="4" t="n"/>
       <c r="M67" s="4" t="n"/>
-      <c r="N67" s="4" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="4" t="n"/>
@@ -2283,7 +2187,6 @@
       <c r="K68" s="4" t="n"/>
       <c r="L68" s="4" t="n"/>
       <c r="M68" s="4" t="n"/>
-      <c r="N68" s="4" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="4" t="n"/>
@@ -2299,7 +2202,6 @@
       <c r="K69" s="4" t="n"/>
       <c r="L69" s="4" t="n"/>
       <c r="M69" s="4" t="n"/>
-      <c r="N69" s="4" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="n"/>
@@ -2315,7 +2217,6 @@
       <c r="K70" s="4" t="n"/>
       <c r="L70" s="4" t="n"/>
       <c r="M70" s="4" t="n"/>
-      <c r="N70" s="4" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="n"/>
@@ -2331,7 +2232,6 @@
       <c r="K71" s="4" t="n"/>
       <c r="L71" s="4" t="n"/>
       <c r="M71" s="4" t="n"/>
-      <c r="N71" s="4" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="n"/>
@@ -2347,7 +2247,6 @@
       <c r="K72" s="4" t="n"/>
       <c r="L72" s="4" t="n"/>
       <c r="M72" s="4" t="n"/>
-      <c r="N72" s="4" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="n"/>
@@ -2363,7 +2262,6 @@
       <c r="K73" s="4" t="n"/>
       <c r="L73" s="4" t="n"/>
       <c r="M73" s="4" t="n"/>
-      <c r="N73" s="4" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="n"/>
@@ -2379,7 +2277,6 @@
       <c r="K74" s="4" t="n"/>
       <c r="L74" s="4" t="n"/>
       <c r="M74" s="4" t="n"/>
-      <c r="N74" s="4" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="4" t="n"/>
@@ -2395,7 +2292,6 @@
       <c r="K75" s="4" t="n"/>
       <c r="L75" s="4" t="n"/>
       <c r="M75" s="4" t="n"/>
-      <c r="N75" s="4" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="4" t="n"/>
@@ -2411,7 +2307,6 @@
       <c r="K76" s="4" t="n"/>
       <c r="L76" s="4" t="n"/>
       <c r="M76" s="4" t="n"/>
-      <c r="N76" s="4" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="4" t="n"/>
@@ -2427,7 +2322,6 @@
       <c r="K77" s="4" t="n"/>
       <c r="L77" s="4" t="n"/>
       <c r="M77" s="4" t="n"/>
-      <c r="N77" s="4" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="4" t="n"/>
@@ -2443,7 +2337,6 @@
       <c r="K78" s="4" t="n"/>
       <c r="L78" s="4" t="n"/>
       <c r="M78" s="4" t="n"/>
-      <c r="N78" s="4" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="4" t="n"/>
@@ -2459,7 +2352,6 @@
       <c r="K79" s="4" t="n"/>
       <c r="L79" s="4" t="n"/>
       <c r="M79" s="4" t="n"/>
-      <c r="N79" s="4" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="4" t="n"/>
@@ -2475,7 +2367,6 @@
       <c r="K80" s="4" t="n"/>
       <c r="L80" s="4" t="n"/>
       <c r="M80" s="4" t="n"/>
-      <c r="N80" s="4" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="4" t="n"/>
@@ -2491,7 +2382,6 @@
       <c r="K81" s="4" t="n"/>
       <c r="L81" s="4" t="n"/>
       <c r="M81" s="4" t="n"/>
-      <c r="N81" s="4" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="4" t="n"/>
@@ -2507,7 +2397,6 @@
       <c r="K82" s="4" t="n"/>
       <c r="L82" s="4" t="n"/>
       <c r="M82" s="4" t="n"/>
-      <c r="N82" s="4" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="4" t="n"/>
@@ -2523,7 +2412,6 @@
       <c r="K83" s="4" t="n"/>
       <c r="L83" s="4" t="n"/>
       <c r="M83" s="4" t="n"/>
-      <c r="N83" s="4" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="4" t="n"/>
@@ -2539,7 +2427,6 @@
       <c r="K84" s="4" t="n"/>
       <c r="L84" s="4" t="n"/>
       <c r="M84" s="4" t="n"/>
-      <c r="N84" s="4" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="4" t="n"/>
@@ -2555,7 +2442,6 @@
       <c r="K85" s="4" t="n"/>
       <c r="L85" s="4" t="n"/>
       <c r="M85" s="4" t="n"/>
-      <c r="N85" s="4" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="4" t="n"/>
@@ -2571,7 +2457,6 @@
       <c r="K86" s="4" t="n"/>
       <c r="L86" s="4" t="n"/>
       <c r="M86" s="4" t="n"/>
-      <c r="N86" s="4" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="4" t="n"/>
@@ -2587,7 +2472,6 @@
       <c r="K87" s="4" t="n"/>
       <c r="L87" s="4" t="n"/>
       <c r="M87" s="4" t="n"/>
-      <c r="N87" s="4" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="4" t="n"/>
@@ -2603,7 +2487,6 @@
       <c r="K88" s="4" t="n"/>
       <c r="L88" s="4" t="n"/>
       <c r="M88" s="4" t="n"/>
-      <c r="N88" s="4" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="4" t="n"/>
@@ -2619,7 +2502,6 @@
       <c r="K89" s="4" t="n"/>
       <c r="L89" s="4" t="n"/>
       <c r="M89" s="4" t="n"/>
-      <c r="N89" s="4" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="n"/>
@@ -2635,7 +2517,6 @@
       <c r="K90" s="4" t="n"/>
       <c r="L90" s="4" t="n"/>
       <c r="M90" s="4" t="n"/>
-      <c r="N90" s="4" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="4" t="n"/>
@@ -2651,7 +2532,6 @@
       <c r="K91" s="4" t="n"/>
       <c r="L91" s="4" t="n"/>
       <c r="M91" s="4" t="n"/>
-      <c r="N91" s="4" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="n"/>
@@ -2667,7 +2547,6 @@
       <c r="K92" s="4" t="n"/>
       <c r="L92" s="4" t="n"/>
       <c r="M92" s="4" t="n"/>
-      <c r="N92" s="4" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="4" t="n"/>
@@ -2683,7 +2562,6 @@
       <c r="K93" s="4" t="n"/>
       <c r="L93" s="4" t="n"/>
       <c r="M93" s="4" t="n"/>
-      <c r="N93" s="4" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="4" t="n"/>
@@ -2699,7 +2577,6 @@
       <c r="K94" s="4" t="n"/>
       <c r="L94" s="4" t="n"/>
       <c r="M94" s="4" t="n"/>
-      <c r="N94" s="4" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="4" t="n"/>
@@ -2715,7 +2592,6 @@
       <c r="K95" s="4" t="n"/>
       <c r="L95" s="4" t="n"/>
       <c r="M95" s="4" t="n"/>
-      <c r="N95" s="4" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="4" t="n"/>
@@ -2731,7 +2607,6 @@
       <c r="K96" s="4" t="n"/>
       <c r="L96" s="4" t="n"/>
       <c r="M96" s="4" t="n"/>
-      <c r="N96" s="4" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="n"/>
@@ -2747,7 +2622,6 @@
       <c r="K97" s="4" t="n"/>
       <c r="L97" s="4" t="n"/>
       <c r="M97" s="4" t="n"/>
-      <c r="N97" s="4" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="4" t="n"/>
@@ -2763,7 +2637,6 @@
       <c r="K98" s="4" t="n"/>
       <c r="L98" s="4" t="n"/>
       <c r="M98" s="4" t="n"/>
-      <c r="N98" s="4" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="4" t="n"/>
@@ -2779,7 +2652,6 @@
       <c r="K99" s="4" t="n"/>
       <c r="L99" s="4" t="n"/>
       <c r="M99" s="4" t="n"/>
-      <c r="N99" s="4" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="4" t="n"/>
@@ -2795,7 +2667,6 @@
       <c r="K100" s="4" t="n"/>
       <c r="L100" s="4" t="n"/>
       <c r="M100" s="4" t="n"/>
-      <c r="N100" s="4" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="n"/>
@@ -2811,7 +2682,6 @@
       <c r="K101" s="4" t="n"/>
       <c r="L101" s="4" t="n"/>
       <c r="M101" s="4" t="n"/>
-      <c r="N101" s="4" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="4" t="n"/>
@@ -2827,7 +2697,6 @@
       <c r="K102" s="4" t="n"/>
       <c r="L102" s="4" t="n"/>
       <c r="M102" s="4" t="n"/>
-      <c r="N102" s="4" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="n"/>
@@ -2843,7 +2712,6 @@
       <c r="K103" s="4" t="n"/>
       <c r="L103" s="4" t="n"/>
       <c r="M103" s="4" t="n"/>
-      <c r="N103" s="4" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="4" t="n"/>
@@ -2859,7 +2727,6 @@
       <c r="K104" s="4" t="n"/>
       <c r="L104" s="4" t="n"/>
       <c r="M104" s="4" t="n"/>
-      <c r="N104" s="4" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="n"/>
@@ -2875,7 +2742,6 @@
       <c r="K105" s="4" t="n"/>
       <c r="L105" s="4" t="n"/>
       <c r="M105" s="4" t="n"/>
-      <c r="N105" s="4" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="4" t="n"/>
@@ -2891,7 +2757,6 @@
       <c r="K106" s="4" t="n"/>
       <c r="L106" s="4" t="n"/>
       <c r="M106" s="4" t="n"/>
-      <c r="N106" s="4" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="4" t="n"/>
@@ -2907,7 +2772,6 @@
       <c r="K107" s="4" t="n"/>
       <c r="L107" s="4" t="n"/>
       <c r="M107" s="4" t="n"/>
-      <c r="N107" s="4" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="4" t="n"/>
@@ -2923,7 +2787,6 @@
       <c r="K108" s="4" t="n"/>
       <c r="L108" s="4" t="n"/>
       <c r="M108" s="4" t="n"/>
-      <c r="N108" s="4" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="4" t="n"/>
@@ -2939,7 +2802,6 @@
       <c r="K109" s="4" t="n"/>
       <c r="L109" s="4" t="n"/>
       <c r="M109" s="4" t="n"/>
-      <c r="N109" s="4" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="4" t="n"/>
@@ -2955,7 +2817,6 @@
       <c r="K110" s="4" t="n"/>
       <c r="L110" s="4" t="n"/>
       <c r="M110" s="4" t="n"/>
-      <c r="N110" s="4" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="4" t="n"/>
@@ -2971,7 +2832,6 @@
       <c r="K111" s="4" t="n"/>
       <c r="L111" s="4" t="n"/>
       <c r="M111" s="4" t="n"/>
-      <c r="N111" s="4" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="4" t="n"/>
@@ -2987,7 +2847,6 @@
       <c r="K112" s="4" t="n"/>
       <c r="L112" s="4" t="n"/>
       <c r="M112" s="4" t="n"/>
-      <c r="N112" s="4" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="4" t="n"/>
@@ -3003,7 +2862,6 @@
       <c r="K113" s="4" t="n"/>
       <c r="L113" s="4" t="n"/>
       <c r="M113" s="4" t="n"/>
-      <c r="N113" s="4" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="4" t="n"/>
@@ -3019,7 +2877,6 @@
       <c r="K114" s="4" t="n"/>
       <c r="L114" s="4" t="n"/>
       <c r="M114" s="4" t="n"/>
-      <c r="N114" s="4" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="n"/>
@@ -3035,7 +2892,6 @@
       <c r="K115" s="4" t="n"/>
       <c r="L115" s="4" t="n"/>
       <c r="M115" s="4" t="n"/>
-      <c r="N115" s="4" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="4" t="n"/>
@@ -3051,7 +2907,6 @@
       <c r="K116" s="4" t="n"/>
       <c r="L116" s="4" t="n"/>
       <c r="M116" s="4" t="n"/>
-      <c r="N116" s="4" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="4" t="n"/>
@@ -3067,7 +2922,6 @@
       <c r="K117" s="4" t="n"/>
       <c r="L117" s="4" t="n"/>
       <c r="M117" s="4" t="n"/>
-      <c r="N117" s="4" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="4" t="n"/>
@@ -3083,7 +2937,6 @@
       <c r="K118" s="4" t="n"/>
       <c r="L118" s="4" t="n"/>
       <c r="M118" s="4" t="n"/>
-      <c r="N118" s="4" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="n"/>
@@ -3099,7 +2952,6 @@
       <c r="K119" s="4" t="n"/>
       <c r="L119" s="4" t="n"/>
       <c r="M119" s="4" t="n"/>
-      <c r="N119" s="4" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="4" t="n"/>
@@ -3115,7 +2967,6 @@
       <c r="K120" s="4" t="n"/>
       <c r="L120" s="4" t="n"/>
       <c r="M120" s="4" t="n"/>
-      <c r="N120" s="4" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="4" t="n"/>
@@ -3131,7 +2982,6 @@
       <c r="K121" s="4" t="n"/>
       <c r="L121" s="4" t="n"/>
       <c r="M121" s="4" t="n"/>
-      <c r="N121" s="4" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="4" t="n"/>
@@ -3147,7 +2997,6 @@
       <c r="K122" s="4" t="n"/>
       <c r="L122" s="4" t="n"/>
       <c r="M122" s="4" t="n"/>
-      <c r="N122" s="4" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="4" t="n"/>
@@ -3163,7 +3012,6 @@
       <c r="K123" s="4" t="n"/>
       <c r="L123" s="4" t="n"/>
       <c r="M123" s="4" t="n"/>
-      <c r="N123" s="4" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="n"/>
@@ -3179,7 +3027,6 @@
       <c r="K124" s="4" t="n"/>
       <c r="L124" s="4" t="n"/>
       <c r="M124" s="4" t="n"/>
-      <c r="N124" s="4" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="4" t="n"/>
@@ -3195,7 +3042,6 @@
       <c r="K125" s="4" t="n"/>
       <c r="L125" s="4" t="n"/>
       <c r="M125" s="4" t="n"/>
-      <c r="N125" s="4" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="4" t="n"/>
@@ -3211,7 +3057,6 @@
       <c r="K126" s="4" t="n"/>
       <c r="L126" s="4" t="n"/>
       <c r="M126" s="4" t="n"/>
-      <c r="N126" s="4" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="4" t="n"/>
@@ -3227,7 +3072,6 @@
       <c r="K127" s="4" t="n"/>
       <c r="L127" s="4" t="n"/>
       <c r="M127" s="4" t="n"/>
-      <c r="N127" s="4" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="4" t="n"/>
@@ -3243,7 +3087,6 @@
       <c r="K128" s="4" t="n"/>
       <c r="L128" s="4" t="n"/>
       <c r="M128" s="4" t="n"/>
-      <c r="N128" s="4" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="4" t="n"/>
@@ -3259,7 +3102,6 @@
       <c r="K129" s="4" t="n"/>
       <c r="L129" s="4" t="n"/>
       <c r="M129" s="4" t="n"/>
-      <c r="N129" s="4" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="4" t="n"/>
@@ -3275,7 +3117,6 @@
       <c r="K130" s="4" t="n"/>
       <c r="L130" s="4" t="n"/>
       <c r="M130" s="4" t="n"/>
-      <c r="N130" s="4" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="4" t="n"/>
@@ -3291,7 +3132,6 @@
       <c r="K131" s="4" t="n"/>
       <c r="L131" s="4" t="n"/>
       <c r="M131" s="4" t="n"/>
-      <c r="N131" s="4" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="4" t="n"/>
@@ -3307,7 +3147,6 @@
       <c r="K132" s="4" t="n"/>
       <c r="L132" s="4" t="n"/>
       <c r="M132" s="4" t="n"/>
-      <c r="N132" s="4" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="4" t="n"/>
@@ -3323,7 +3162,6 @@
       <c r="K133" s="4" t="n"/>
       <c r="L133" s="4" t="n"/>
       <c r="M133" s="4" t="n"/>
-      <c r="N133" s="4" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="4" t="n"/>
@@ -3339,7 +3177,6 @@
       <c r="K134" s="4" t="n"/>
       <c r="L134" s="4" t="n"/>
       <c r="M134" s="4" t="n"/>
-      <c r="N134" s="4" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="4" t="n"/>
@@ -3355,7 +3192,6 @@
       <c r="K135" s="4" t="n"/>
       <c r="L135" s="4" t="n"/>
       <c r="M135" s="4" t="n"/>
-      <c r="N135" s="4" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="4" t="n"/>
@@ -3371,7 +3207,6 @@
       <c r="K136" s="4" t="n"/>
       <c r="L136" s="4" t="n"/>
       <c r="M136" s="4" t="n"/>
-      <c r="N136" s="4" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="4" t="n"/>
@@ -3387,7 +3222,6 @@
       <c r="K137" s="4" t="n"/>
       <c r="L137" s="4" t="n"/>
       <c r="M137" s="4" t="n"/>
-      <c r="N137" s="4" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="4" t="n"/>
@@ -3403,7 +3237,6 @@
       <c r="K138" s="4" t="n"/>
       <c r="L138" s="4" t="n"/>
       <c r="M138" s="4" t="n"/>
-      <c r="N138" s="4" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="4" t="n"/>
@@ -3419,7 +3252,6 @@
       <c r="K139" s="4" t="n"/>
       <c r="L139" s="4" t="n"/>
       <c r="M139" s="4" t="n"/>
-      <c r="N139" s="4" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="4" t="n"/>
@@ -3435,7 +3267,6 @@
       <c r="K140" s="4" t="n"/>
       <c r="L140" s="4" t="n"/>
       <c r="M140" s="4" t="n"/>
-      <c r="N140" s="4" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="n"/>
@@ -3451,7 +3282,6 @@
       <c r="K141" s="4" t="n"/>
       <c r="L141" s="4" t="n"/>
       <c r="M141" s="4" t="n"/>
-      <c r="N141" s="4" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="4" t="n"/>
@@ -3467,7 +3297,6 @@
       <c r="K142" s="4" t="n"/>
       <c r="L142" s="4" t="n"/>
       <c r="M142" s="4" t="n"/>
-      <c r="N142" s="4" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="n"/>
@@ -3483,7 +3312,6 @@
       <c r="K143" s="4" t="n"/>
       <c r="L143" s="4" t="n"/>
       <c r="M143" s="4" t="n"/>
-      <c r="N143" s="4" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="4" t="n"/>
@@ -3499,7 +3327,6 @@
       <c r="K144" s="4" t="n"/>
       <c r="L144" s="4" t="n"/>
       <c r="M144" s="4" t="n"/>
-      <c r="N144" s="4" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="4" t="n"/>
@@ -3515,7 +3342,6 @@
       <c r="K145" s="4" t="n"/>
       <c r="L145" s="4" t="n"/>
       <c r="M145" s="4" t="n"/>
-      <c r="N145" s="4" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="n"/>
@@ -3531,7 +3357,6 @@
       <c r="K146" s="4" t="n"/>
       <c r="L146" s="4" t="n"/>
       <c r="M146" s="4" t="n"/>
-      <c r="N146" s="4" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="4" t="n"/>
@@ -3547,7 +3372,6 @@
       <c r="K147" s="4" t="n"/>
       <c r="L147" s="4" t="n"/>
       <c r="M147" s="4" t="n"/>
-      <c r="N147" s="4" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="4" t="n"/>
@@ -3563,7 +3387,6 @@
       <c r="K148" s="4" t="n"/>
       <c r="L148" s="4" t="n"/>
       <c r="M148" s="4" t="n"/>
-      <c r="N148" s="4" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="4" t="n"/>
@@ -3579,7 +3402,6 @@
       <c r="K149" s="4" t="n"/>
       <c r="L149" s="4" t="n"/>
       <c r="M149" s="4" t="n"/>
-      <c r="N149" s="4" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="4" t="n"/>
@@ -3595,7 +3417,6 @@
       <c r="K150" s="4" t="n"/>
       <c r="L150" s="4" t="n"/>
       <c r="M150" s="4" t="n"/>
-      <c r="N150" s="4" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="4" t="n"/>
@@ -3611,7 +3432,6 @@
       <c r="K151" s="4" t="n"/>
       <c r="L151" s="4" t="n"/>
       <c r="M151" s="4" t="n"/>
-      <c r="N151" s="4" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="4" t="n"/>
@@ -3627,7 +3447,6 @@
       <c r="K152" s="4" t="n"/>
       <c r="L152" s="4" t="n"/>
       <c r="M152" s="4" t="n"/>
-      <c r="N152" s="4" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="4" t="n"/>
@@ -3643,7 +3462,6 @@
       <c r="K153" s="4" t="n"/>
       <c r="L153" s="4" t="n"/>
       <c r="M153" s="4" t="n"/>
-      <c r="N153" s="4" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="4" t="n"/>
@@ -3659,7 +3477,6 @@
       <c r="K154" s="4" t="n"/>
       <c r="L154" s="4" t="n"/>
       <c r="M154" s="4" t="n"/>
-      <c r="N154" s="4" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="n"/>
@@ -3675,7 +3492,6 @@
       <c r="K155" s="4" t="n"/>
       <c r="L155" s="4" t="n"/>
       <c r="M155" s="4" t="n"/>
-      <c r="N155" s="4" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="4" t="n"/>
@@ -3691,7 +3507,6 @@
       <c r="K156" s="4" t="n"/>
       <c r="L156" s="4" t="n"/>
       <c r="M156" s="4" t="n"/>
-      <c r="N156" s="4" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="4" t="n"/>
@@ -3707,7 +3522,6 @@
       <c r="K157" s="4" t="n"/>
       <c r="L157" s="4" t="n"/>
       <c r="M157" s="4" t="n"/>
-      <c r="N157" s="4" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="4" t="n"/>
@@ -3723,7 +3537,6 @@
       <c r="K158" s="4" t="n"/>
       <c r="L158" s="4" t="n"/>
       <c r="M158" s="4" t="n"/>
-      <c r="N158" s="4" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="4" t="n"/>
@@ -3739,7 +3552,6 @@
       <c r="K159" s="4" t="n"/>
       <c r="L159" s="4" t="n"/>
       <c r="M159" s="4" t="n"/>
-      <c r="N159" s="4" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="4" t="n"/>
@@ -3755,7 +3567,6 @@
       <c r="K160" s="4" t="n"/>
       <c r="L160" s="4" t="n"/>
       <c r="M160" s="4" t="n"/>
-      <c r="N160" s="4" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="4" t="n"/>
@@ -3771,7 +3582,6 @@
       <c r="K161" s="4" t="n"/>
       <c r="L161" s="4" t="n"/>
       <c r="M161" s="4" t="n"/>
-      <c r="N161" s="4" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="4" t="n"/>
@@ -3787,7 +3597,6 @@
       <c r="K162" s="4" t="n"/>
       <c r="L162" s="4" t="n"/>
       <c r="M162" s="4" t="n"/>
-      <c r="N162" s="4" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="4" t="n"/>
@@ -3803,7 +3612,6 @@
       <c r="K163" s="4" t="n"/>
       <c r="L163" s="4" t="n"/>
       <c r="M163" s="4" t="n"/>
-      <c r="N163" s="4" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="4" t="n"/>
@@ -3819,7 +3627,6 @@
       <c r="K164" s="4" t="n"/>
       <c r="L164" s="4" t="n"/>
       <c r="M164" s="4" t="n"/>
-      <c r="N164" s="4" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="4" t="n"/>
@@ -3835,7 +3642,6 @@
       <c r="K165" s="4" t="n"/>
       <c r="L165" s="4" t="n"/>
       <c r="M165" s="4" t="n"/>
-      <c r="N165" s="4" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="4" t="n"/>
@@ -3851,7 +3657,6 @@
       <c r="K166" s="4" t="n"/>
       <c r="L166" s="4" t="n"/>
       <c r="M166" s="4" t="n"/>
-      <c r="N166" s="4" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="4" t="n"/>
@@ -3867,7 +3672,6 @@
       <c r="K167" s="4" t="n"/>
       <c r="L167" s="4" t="n"/>
       <c r="M167" s="4" t="n"/>
-      <c r="N167" s="4" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="4" t="n"/>
@@ -3883,7 +3687,6 @@
       <c r="K168" s="4" t="n"/>
       <c r="L168" s="4" t="n"/>
       <c r="M168" s="4" t="n"/>
-      <c r="N168" s="4" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="4" t="n"/>
@@ -3899,7 +3702,6 @@
       <c r="K169" s="4" t="n"/>
       <c r="L169" s="4" t="n"/>
       <c r="M169" s="4" t="n"/>
-      <c r="N169" s="4" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="4" t="n"/>
@@ -3915,7 +3717,6 @@
       <c r="K170" s="4" t="n"/>
       <c r="L170" s="4" t="n"/>
       <c r="M170" s="4" t="n"/>
-      <c r="N170" s="4" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="4" t="n"/>
@@ -3931,7 +3732,6 @@
       <c r="K171" s="4" t="n"/>
       <c r="L171" s="4" t="n"/>
       <c r="M171" s="4" t="n"/>
-      <c r="N171" s="4" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="4" t="n"/>
@@ -3947,7 +3747,6 @@
       <c r="K172" s="4" t="n"/>
       <c r="L172" s="4" t="n"/>
       <c r="M172" s="4" t="n"/>
-      <c r="N172" s="4" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="4" t="n"/>
@@ -3963,7 +3762,6 @@
       <c r="K173" s="4" t="n"/>
       <c r="L173" s="4" t="n"/>
       <c r="M173" s="4" t="n"/>
-      <c r="N173" s="4" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="4" t="n"/>
@@ -3979,7 +3777,6 @@
       <c r="K174" s="4" t="n"/>
       <c r="L174" s="4" t="n"/>
       <c r="M174" s="4" t="n"/>
-      <c r="N174" s="4" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="4" t="n"/>
@@ -3995,7 +3792,6 @@
       <c r="K175" s="4" t="n"/>
       <c r="L175" s="4" t="n"/>
       <c r="M175" s="4" t="n"/>
-      <c r="N175" s="4" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="4" t="n"/>
@@ -4011,7 +3807,6 @@
       <c r="K176" s="4" t="n"/>
       <c r="L176" s="4" t="n"/>
       <c r="M176" s="4" t="n"/>
-      <c r="N176" s="4" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="4" t="n"/>
@@ -4027,7 +3822,6 @@
       <c r="K177" s="4" t="n"/>
       <c r="L177" s="4" t="n"/>
       <c r="M177" s="4" t="n"/>
-      <c r="N177" s="4" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="4" t="n"/>
@@ -4043,7 +3837,6 @@
       <c r="K178" s="4" t="n"/>
       <c r="L178" s="4" t="n"/>
       <c r="M178" s="4" t="n"/>
-      <c r="N178" s="4" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="4" t="n"/>
@@ -4059,7 +3852,6 @@
       <c r="K179" s="4" t="n"/>
       <c r="L179" s="4" t="n"/>
       <c r="M179" s="4" t="n"/>
-      <c r="N179" s="4" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="4" t="n"/>
@@ -4075,7 +3867,6 @@
       <c r="K180" s="4" t="n"/>
       <c r="L180" s="4" t="n"/>
       <c r="M180" s="4" t="n"/>
-      <c r="N180" s="4" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="4" t="n"/>
@@ -4091,7 +3882,6 @@
       <c r="K181" s="4" t="n"/>
       <c r="L181" s="4" t="n"/>
       <c r="M181" s="4" t="n"/>
-      <c r="N181" s="4" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="4" t="n"/>
@@ -4107,7 +3897,6 @@
       <c r="K182" s="4" t="n"/>
       <c r="L182" s="4" t="n"/>
       <c r="M182" s="4" t="n"/>
-      <c r="N182" s="4" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="4" t="n"/>
@@ -4123,7 +3912,6 @@
       <c r="K183" s="4" t="n"/>
       <c r="L183" s="4" t="n"/>
       <c r="M183" s="4" t="n"/>
-      <c r="N183" s="4" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="4" t="n"/>
@@ -4139,7 +3927,6 @@
       <c r="K184" s="4" t="n"/>
       <c r="L184" s="4" t="n"/>
       <c r="M184" s="4" t="n"/>
-      <c r="N184" s="4" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="4" t="n"/>
@@ -4155,7 +3942,6 @@
       <c r="K185" s="4" t="n"/>
       <c r="L185" s="4" t="n"/>
       <c r="M185" s="4" t="n"/>
-      <c r="N185" s="4" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="4" t="n"/>
@@ -4171,7 +3957,6 @@
       <c r="K186" s="4" t="n"/>
       <c r="L186" s="4" t="n"/>
       <c r="M186" s="4" t="n"/>
-      <c r="N186" s="4" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="4" t="n"/>
@@ -4187,7 +3972,6 @@
       <c r="K187" s="4" t="n"/>
       <c r="L187" s="4" t="n"/>
       <c r="M187" s="4" t="n"/>
-      <c r="N187" s="4" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="4" t="n"/>
@@ -4203,7 +3987,6 @@
       <c r="K188" s="4" t="n"/>
       <c r="L188" s="4" t="n"/>
       <c r="M188" s="4" t="n"/>
-      <c r="N188" s="4" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="4" t="n"/>
@@ -4219,7 +4002,6 @@
       <c r="K189" s="4" t="n"/>
       <c r="L189" s="4" t="n"/>
       <c r="M189" s="4" t="n"/>
-      <c r="N189" s="4" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="4" t="n"/>
@@ -4235,7 +4017,6 @@
       <c r="K190" s="4" t="n"/>
       <c r="L190" s="4" t="n"/>
       <c r="M190" s="4" t="n"/>
-      <c r="N190" s="4" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="4" t="n"/>
@@ -4251,7 +4032,6 @@
       <c r="K191" s="4" t="n"/>
       <c r="L191" s="4" t="n"/>
       <c r="M191" s="4" t="n"/>
-      <c r="N191" s="4" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="4" t="n"/>
@@ -4267,7 +4047,6 @@
       <c r="K192" s="4" t="n"/>
       <c r="L192" s="4" t="n"/>
       <c r="M192" s="4" t="n"/>
-      <c r="N192" s="4" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="4" t="n"/>
@@ -4283,7 +4062,6 @@
       <c r="K193" s="4" t="n"/>
       <c r="L193" s="4" t="n"/>
       <c r="M193" s="4" t="n"/>
-      <c r="N193" s="4" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="4" t="n"/>
@@ -4299,7 +4077,6 @@
       <c r="K194" s="4" t="n"/>
       <c r="L194" s="4" t="n"/>
       <c r="M194" s="4" t="n"/>
-      <c r="N194" s="4" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="4" t="n"/>
@@ -4315,7 +4092,6 @@
       <c r="K195" s="4" t="n"/>
       <c r="L195" s="4" t="n"/>
       <c r="M195" s="4" t="n"/>
-      <c r="N195" s="4" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="4" t="n"/>
@@ -4331,7 +4107,6 @@
       <c r="K196" s="4" t="n"/>
       <c r="L196" s="4" t="n"/>
       <c r="M196" s="4" t="n"/>
-      <c r="N196" s="4" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="4" t="n"/>
@@ -4347,7 +4122,6 @@
       <c r="K197" s="4" t="n"/>
       <c r="L197" s="4" t="n"/>
       <c r="M197" s="4" t="n"/>
-      <c r="N197" s="4" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="4" t="n"/>
@@ -4363,7 +4137,6 @@
       <c r="K198" s="4" t="n"/>
       <c r="L198" s="4" t="n"/>
       <c r="M198" s="4" t="n"/>
-      <c r="N198" s="4" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="4" t="n"/>
@@ -4379,7 +4152,6 @@
       <c r="K199" s="4" t="n"/>
       <c r="L199" s="4" t="n"/>
       <c r="M199" s="4" t="n"/>
-      <c r="N199" s="4" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="4" t="n"/>
@@ -4395,7 +4167,6 @@
       <c r="K200" s="4" t="n"/>
       <c r="L200" s="4" t="n"/>
       <c r="M200" s="4" t="n"/>
-      <c r="N200" s="4" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="4" t="n"/>
@@ -4411,7 +4182,6 @@
       <c r="K201" s="4" t="n"/>
       <c r="L201" s="4" t="n"/>
       <c r="M201" s="4" t="n"/>
-      <c r="N201" s="4" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="4" t="n"/>
@@ -4427,7 +4197,6 @@
       <c r="K202" s="4" t="n"/>
       <c r="L202" s="4" t="n"/>
       <c r="M202" s="4" t="n"/>
-      <c r="N202" s="4" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="4" t="n"/>
@@ -4443,7 +4212,6 @@
       <c r="K203" s="4" t="n"/>
       <c r="L203" s="4" t="n"/>
       <c r="M203" s="4" t="n"/>
-      <c r="N203" s="4" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="4" t="n"/>
@@ -4459,7 +4227,6 @@
       <c r="K204" s="4" t="n"/>
       <c r="L204" s="4" t="n"/>
       <c r="M204" s="4" t="n"/>
-      <c r="N204" s="4" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="4" t="n"/>
@@ -4475,7 +4242,6 @@
       <c r="K205" s="4" t="n"/>
       <c r="L205" s="4" t="n"/>
       <c r="M205" s="4" t="n"/>
-      <c r="N205" s="4" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="4" t="n"/>
@@ -4491,7 +4257,6 @@
       <c r="K206" s="4" t="n"/>
       <c r="L206" s="4" t="n"/>
       <c r="M206" s="4" t="n"/>
-      <c r="N206" s="4" t="n"/>
     </row>
     <row r="207">
       <c r="A207" s="4" t="n"/>
@@ -4507,7 +4272,6 @@
       <c r="K207" s="4" t="n"/>
       <c r="L207" s="4" t="n"/>
       <c r="M207" s="4" t="n"/>
-      <c r="N207" s="4" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="4" t="n"/>
@@ -4523,7 +4287,6 @@
       <c r="K208" s="4" t="n"/>
       <c r="L208" s="4" t="n"/>
       <c r="M208" s="4" t="n"/>
-      <c r="N208" s="4" t="n"/>
     </row>
     <row r="209">
       <c r="A209" s="4" t="n"/>
@@ -4539,7 +4302,6 @@
       <c r="K209" s="4" t="n"/>
       <c r="L209" s="4" t="n"/>
       <c r="M209" s="4" t="n"/>
-      <c r="N209" s="4" t="n"/>
     </row>
     <row r="210">
       <c r="A210" s="4" t="n"/>
@@ -4555,7 +4317,6 @@
       <c r="K210" s="4" t="n"/>
       <c r="L210" s="4" t="n"/>
       <c r="M210" s="4" t="n"/>
-      <c r="N210" s="4" t="n"/>
     </row>
     <row r="211">
       <c r="A211" s="4" t="n"/>
@@ -4571,7 +4332,6 @@
       <c r="K211" s="4" t="n"/>
       <c r="L211" s="4" t="n"/>
       <c r="M211" s="4" t="n"/>
-      <c r="N211" s="4" t="n"/>
     </row>
     <row r="212">
       <c r="A212" s="4" t="n"/>
@@ -4587,7 +4347,6 @@
       <c r="K212" s="4" t="n"/>
       <c r="L212" s="4" t="n"/>
       <c r="M212" s="4" t="n"/>
-      <c r="N212" s="4" t="n"/>
     </row>
     <row r="213">
       <c r="A213" s="4" t="n"/>
@@ -4603,7 +4362,6 @@
       <c r="K213" s="4" t="n"/>
       <c r="L213" s="4" t="n"/>
       <c r="M213" s="4" t="n"/>
-      <c r="N213" s="4" t="n"/>
     </row>
     <row r="214">
       <c r="A214" s="4" t="n"/>
@@ -4619,7 +4377,6 @@
       <c r="K214" s="4" t="n"/>
       <c r="L214" s="4" t="n"/>
       <c r="M214" s="4" t="n"/>
-      <c r="N214" s="4" t="n"/>
     </row>
     <row r="215">
       <c r="A215" s="4" t="n"/>
@@ -4635,7 +4392,6 @@
       <c r="K215" s="4" t="n"/>
       <c r="L215" s="4" t="n"/>
       <c r="M215" s="4" t="n"/>
-      <c r="N215" s="4" t="n"/>
     </row>
     <row r="216">
       <c r="A216" s="4" t="n"/>
@@ -4651,7 +4407,6 @@
       <c r="K216" s="4" t="n"/>
       <c r="L216" s="4" t="n"/>
       <c r="M216" s="4" t="n"/>
-      <c r="N216" s="4" t="n"/>
     </row>
     <row r="217">
       <c r="A217" s="4" t="n"/>
@@ -4667,7 +4422,6 @@
       <c r="K217" s="4" t="n"/>
       <c r="L217" s="4" t="n"/>
       <c r="M217" s="4" t="n"/>
-      <c r="N217" s="4" t="n"/>
     </row>
     <row r="218">
       <c r="A218" s="4" t="n"/>
@@ -4683,7 +4437,6 @@
       <c r="K218" s="4" t="n"/>
       <c r="L218" s="4" t="n"/>
       <c r="M218" s="4" t="n"/>
-      <c r="N218" s="4" t="n"/>
     </row>
     <row r="219">
       <c r="A219" s="4" t="n"/>
@@ -4699,7 +4452,6 @@
       <c r="K219" s="4" t="n"/>
       <c r="L219" s="4" t="n"/>
       <c r="M219" s="4" t="n"/>
-      <c r="N219" s="4" t="n"/>
     </row>
     <row r="220">
       <c r="A220" s="4" t="n"/>
@@ -4715,7 +4467,6 @@
       <c r="K220" s="4" t="n"/>
       <c r="L220" s="4" t="n"/>
       <c r="M220" s="4" t="n"/>
-      <c r="N220" s="4" t="n"/>
     </row>
     <row r="221">
       <c r="A221" s="4" t="n"/>
@@ -4731,7 +4482,6 @@
       <c r="K221" s="4" t="n"/>
       <c r="L221" s="4" t="n"/>
       <c r="M221" s="4" t="n"/>
-      <c r="N221" s="4" t="n"/>
     </row>
     <row r="222">
       <c r="A222" s="4" t="n"/>
@@ -4747,7 +4497,6 @@
       <c r="K222" s="4" t="n"/>
       <c r="L222" s="4" t="n"/>
       <c r="M222" s="4" t="n"/>
-      <c r="N222" s="4" t="n"/>
     </row>
     <row r="223">
       <c r="A223" s="4" t="n"/>
@@ -4763,7 +4512,6 @@
       <c r="K223" s="4" t="n"/>
       <c r="L223" s="4" t="n"/>
       <c r="M223" s="4" t="n"/>
-      <c r="N223" s="4" t="n"/>
     </row>
     <row r="224">
       <c r="A224" s="4" t="n"/>
@@ -4779,7 +4527,6 @@
       <c r="K224" s="4" t="n"/>
       <c r="L224" s="4" t="n"/>
       <c r="M224" s="4" t="n"/>
-      <c r="N224" s="4" t="n"/>
     </row>
     <row r="225">
       <c r="A225" s="4" t="n"/>
@@ -4795,7 +4542,6 @@
       <c r="K225" s="4" t="n"/>
       <c r="L225" s="4" t="n"/>
       <c r="M225" s="4" t="n"/>
-      <c r="N225" s="4" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="4" t="n"/>
@@ -4811,7 +4557,6 @@
       <c r="K226" s="4" t="n"/>
       <c r="L226" s="4" t="n"/>
       <c r="M226" s="4" t="n"/>
-      <c r="N226" s="4" t="n"/>
     </row>
     <row r="227">
       <c r="A227" s="4" t="n"/>
@@ -4827,7 +4572,6 @@
       <c r="K227" s="4" t="n"/>
       <c r="L227" s="4" t="n"/>
       <c r="M227" s="4" t="n"/>
-      <c r="N227" s="4" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="4" t="n"/>
@@ -4843,7 +4587,6 @@
       <c r="K228" s="4" t="n"/>
       <c r="L228" s="4" t="n"/>
       <c r="M228" s="4" t="n"/>
-      <c r="N228" s="4" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="4" t="n"/>
@@ -4859,7 +4602,6 @@
       <c r="K229" s="4" t="n"/>
       <c r="L229" s="4" t="n"/>
       <c r="M229" s="4" t="n"/>
-      <c r="N229" s="4" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="4" t="n"/>
@@ -4875,7 +4617,6 @@
       <c r="K230" s="4" t="n"/>
       <c r="L230" s="4" t="n"/>
       <c r="M230" s="4" t="n"/>
-      <c r="N230" s="4" t="n"/>
     </row>
     <row r="231">
       <c r="A231" s="4" t="n"/>
@@ -4891,7 +4632,6 @@
       <c r="K231" s="4" t="n"/>
       <c r="L231" s="4" t="n"/>
       <c r="M231" s="4" t="n"/>
-      <c r="N231" s="4" t="n"/>
     </row>
     <row r="232">
       <c r="A232" s="4" t="n"/>
@@ -4907,7 +4647,6 @@
       <c r="K232" s="4" t="n"/>
       <c r="L232" s="4" t="n"/>
       <c r="M232" s="4" t="n"/>
-      <c r="N232" s="4" t="n"/>
     </row>
     <row r="233">
       <c r="A233" s="4" t="n"/>
@@ -4923,7 +4662,6 @@
       <c r="K233" s="4" t="n"/>
       <c r="L233" s="4" t="n"/>
       <c r="M233" s="4" t="n"/>
-      <c r="N233" s="4" t="n"/>
     </row>
     <row r="234">
       <c r="A234" s="4" t="n"/>
@@ -4939,7 +4677,6 @@
       <c r="K234" s="4" t="n"/>
       <c r="L234" s="4" t="n"/>
       <c r="M234" s="4" t="n"/>
-      <c r="N234" s="4" t="n"/>
     </row>
     <row r="235">
       <c r="A235" s="4" t="n"/>
@@ -4955,7 +4692,6 @@
       <c r="K235" s="4" t="n"/>
       <c r="L235" s="4" t="n"/>
       <c r="M235" s="4" t="n"/>
-      <c r="N235" s="4" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="4" t="n"/>
@@ -4971,7 +4707,6 @@
       <c r="K236" s="4" t="n"/>
       <c r="L236" s="4" t="n"/>
       <c r="M236" s="4" t="n"/>
-      <c r="N236" s="4" t="n"/>
     </row>
     <row r="237">
       <c r="A237" s="4" t="n"/>
@@ -4987,7 +4722,6 @@
       <c r="K237" s="4" t="n"/>
       <c r="L237" s="4" t="n"/>
       <c r="M237" s="4" t="n"/>
-      <c r="N237" s="4" t="n"/>
     </row>
     <row r="238">
       <c r="A238" s="4" t="n"/>
@@ -5003,7 +4737,6 @@
       <c r="K238" s="4" t="n"/>
       <c r="L238" s="4" t="n"/>
       <c r="M238" s="4" t="n"/>
-      <c r="N238" s="4" t="n"/>
     </row>
     <row r="239">
       <c r="A239" s="4" t="n"/>
@@ -5019,7 +4752,6 @@
       <c r="K239" s="4" t="n"/>
       <c r="L239" s="4" t="n"/>
       <c r="M239" s="4" t="n"/>
-      <c r="N239" s="4" t="n"/>
     </row>
     <row r="240">
       <c r="A240" s="4" t="n"/>
@@ -5035,7 +4767,6 @@
       <c r="K240" s="4" t="n"/>
       <c r="L240" s="4" t="n"/>
       <c r="M240" s="4" t="n"/>
-      <c r="N240" s="4" t="n"/>
     </row>
     <row r="241">
       <c r="A241" s="4" t="n"/>
@@ -5051,7 +4782,6 @@
       <c r="K241" s="4" t="n"/>
       <c r="L241" s="4" t="n"/>
       <c r="M241" s="4" t="n"/>
-      <c r="N241" s="4" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="4" t="n"/>
@@ -5067,7 +4797,6 @@
       <c r="K242" s="4" t="n"/>
       <c r="L242" s="4" t="n"/>
       <c r="M242" s="4" t="n"/>
-      <c r="N242" s="4" t="n"/>
     </row>
     <row r="243">
       <c r="A243" s="4" t="n"/>
@@ -5083,7 +4812,6 @@
       <c r="K243" s="4" t="n"/>
       <c r="L243" s="4" t="n"/>
       <c r="M243" s="4" t="n"/>
-      <c r="N243" s="4" t="n"/>
     </row>
     <row r="244">
       <c r="A244" s="4" t="n"/>
@@ -5099,7 +4827,6 @@
       <c r="K244" s="4" t="n"/>
       <c r="L244" s="4" t="n"/>
       <c r="M244" s="4" t="n"/>
-      <c r="N244" s="4" t="n"/>
     </row>
     <row r="245">
       <c r="A245" s="4" t="n"/>
@@ -5115,7 +4842,6 @@
       <c r="K245" s="4" t="n"/>
       <c r="L245" s="4" t="n"/>
       <c r="M245" s="4" t="n"/>
-      <c r="N245" s="4" t="n"/>
     </row>
     <row r="246">
       <c r="A246" s="4" t="n"/>
@@ -5131,7 +4857,6 @@
       <c r="K246" s="4" t="n"/>
       <c r="L246" s="4" t="n"/>
       <c r="M246" s="4" t="n"/>
-      <c r="N246" s="4" t="n"/>
     </row>
     <row r="247">
       <c r="A247" s="4" t="n"/>
@@ -5147,7 +4872,6 @@
       <c r="K247" s="4" t="n"/>
       <c r="L247" s="4" t="n"/>
       <c r="M247" s="4" t="n"/>
-      <c r="N247" s="4" t="n"/>
     </row>
     <row r="248">
       <c r="A248" s="4" t="n"/>
@@ -5163,7 +4887,6 @@
       <c r="K248" s="4" t="n"/>
       <c r="L248" s="4" t="n"/>
       <c r="M248" s="4" t="n"/>
-      <c r="N248" s="4" t="n"/>
     </row>
     <row r="249">
       <c r="A249" s="4" t="n"/>
@@ -5179,7 +4902,6 @@
       <c r="K249" s="4" t="n"/>
       <c r="L249" s="4" t="n"/>
       <c r="M249" s="4" t="n"/>
-      <c r="N249" s="4" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="4" t="n"/>
@@ -5195,7 +4917,6 @@
       <c r="K250" s="4" t="n"/>
       <c r="L250" s="4" t="n"/>
       <c r="M250" s="4" t="n"/>
-      <c r="N250" s="4" t="n"/>
     </row>
     <row r="251">
       <c r="A251" s="4" t="n"/>
@@ -5211,7 +4932,6 @@
       <c r="K251" s="4" t="n"/>
       <c r="L251" s="4" t="n"/>
       <c r="M251" s="4" t="n"/>
-      <c r="N251" s="4" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="4" t="n"/>
@@ -5227,7 +4947,6 @@
       <c r="K252" s="4" t="n"/>
       <c r="L252" s="4" t="n"/>
       <c r="M252" s="4" t="n"/>
-      <c r="N252" s="4" t="n"/>
     </row>
     <row r="253">
       <c r="A253" s="4" t="n"/>
@@ -5243,7 +4962,6 @@
       <c r="K253" s="4" t="n"/>
       <c r="L253" s="4" t="n"/>
       <c r="M253" s="4" t="n"/>
-      <c r="N253" s="4" t="n"/>
     </row>
     <row r="254">
       <c r="A254" s="4" t="n"/>
@@ -5259,7 +4977,6 @@
       <c r="K254" s="4" t="n"/>
       <c r="L254" s="4" t="n"/>
       <c r="M254" s="4" t="n"/>
-      <c r="N254" s="4" t="n"/>
     </row>
     <row r="255">
       <c r="A255" s="4" t="n"/>
@@ -5275,7 +4992,6 @@
       <c r="K255" s="4" t="n"/>
       <c r="L255" s="4" t="n"/>
       <c r="M255" s="4" t="n"/>
-      <c r="N255" s="4" t="n"/>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n"/>
@@ -5291,7 +5007,6 @@
       <c r="K256" s="4" t="n"/>
       <c r="L256" s="4" t="n"/>
       <c r="M256" s="4" t="n"/>
-      <c r="N256" s="4" t="n"/>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n"/>
@@ -5307,7 +5022,6 @@
       <c r="K257" s="4" t="n"/>
       <c r="L257" s="4" t="n"/>
       <c r="M257" s="4" t="n"/>
-      <c r="N257" s="4" t="n"/>
     </row>
     <row r="258">
       <c r="A258" s="4" t="n"/>
@@ -5323,7 +5037,6 @@
       <c r="K258" s="4" t="n"/>
       <c r="L258" s="4" t="n"/>
       <c r="M258" s="4" t="n"/>
-      <c r="N258" s="4" t="n"/>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n"/>
@@ -5339,7 +5052,6 @@
       <c r="K259" s="4" t="n"/>
       <c r="L259" s="4" t="n"/>
       <c r="M259" s="4" t="n"/>
-      <c r="N259" s="4" t="n"/>
     </row>
     <row r="260">
       <c r="A260" s="4" t="n"/>
@@ -5355,7 +5067,6 @@
       <c r="K260" s="4" t="n"/>
       <c r="L260" s="4" t="n"/>
       <c r="M260" s="4" t="n"/>
-      <c r="N260" s="4" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n"/>
@@ -5371,7 +5082,6 @@
       <c r="K261" s="4" t="n"/>
       <c r="L261" s="4" t="n"/>
       <c r="M261" s="4" t="n"/>
-      <c r="N261" s="4" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n"/>
@@ -5387,7 +5097,6 @@
       <c r="K262" s="4" t="n"/>
       <c r="L262" s="4" t="n"/>
       <c r="M262" s="4" t="n"/>
-      <c r="N262" s="4" t="n"/>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n"/>
@@ -5403,7 +5112,6 @@
       <c r="K263" s="4" t="n"/>
       <c r="L263" s="4" t="n"/>
       <c r="M263" s="4" t="n"/>
-      <c r="N263" s="4" t="n"/>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n"/>
@@ -5419,7 +5127,6 @@
       <c r="K264" s="4" t="n"/>
       <c r="L264" s="4" t="n"/>
       <c r="M264" s="4" t="n"/>
-      <c r="N264" s="4" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n"/>
@@ -5435,7 +5142,6 @@
       <c r="K265" s="4" t="n"/>
       <c r="L265" s="4" t="n"/>
       <c r="M265" s="4" t="n"/>
-      <c r="N265" s="4" t="n"/>
     </row>
     <row r="266">
       <c r="A266" s="4" t="n"/>
@@ -5451,7 +5157,6 @@
       <c r="K266" s="4" t="n"/>
       <c r="L266" s="4" t="n"/>
       <c r="M266" s="4" t="n"/>
-      <c r="N266" s="4" t="n"/>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n"/>
@@ -5467,7 +5172,6 @@
       <c r="K267" s="4" t="n"/>
       <c r="L267" s="4" t="n"/>
       <c r="M267" s="4" t="n"/>
-      <c r="N267" s="4" t="n"/>
     </row>
     <row r="268">
       <c r="A268" s="4" t="n"/>
@@ -5483,7 +5187,6 @@
       <c r="K268" s="4" t="n"/>
       <c r="L268" s="4" t="n"/>
       <c r="M268" s="4" t="n"/>
-      <c r="N268" s="4" t="n"/>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n"/>
@@ -5499,7 +5202,6 @@
       <c r="K269" s="4" t="n"/>
       <c r="L269" s="4" t="n"/>
       <c r="M269" s="4" t="n"/>
-      <c r="N269" s="4" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n"/>
@@ -5515,7 +5217,6 @@
       <c r="K270" s="4" t="n"/>
       <c r="L270" s="4" t="n"/>
       <c r="M270" s="4" t="n"/>
-      <c r="N270" s="4" t="n"/>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n"/>
@@ -5531,7 +5232,6 @@
       <c r="K271" s="4" t="n"/>
       <c r="L271" s="4" t="n"/>
       <c r="M271" s="4" t="n"/>
-      <c r="N271" s="4" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n"/>
@@ -5547,7 +5247,6 @@
       <c r="K272" s="4" t="n"/>
       <c r="L272" s="4" t="n"/>
       <c r="M272" s="4" t="n"/>
-      <c r="N272" s="4" t="n"/>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n"/>
@@ -5563,7 +5262,6 @@
       <c r="K273" s="4" t="n"/>
       <c r="L273" s="4" t="n"/>
       <c r="M273" s="4" t="n"/>
-      <c r="N273" s="4" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="4" t="n"/>
@@ -5579,7 +5277,6 @@
       <c r="K274" s="4" t="n"/>
       <c r="L274" s="4" t="n"/>
       <c r="M274" s="4" t="n"/>
-      <c r="N274" s="4" t="n"/>
     </row>
     <row r="275">
       <c r="A275" s="4" t="n"/>
@@ -5595,7 +5292,6 @@
       <c r="K275" s="4" t="n"/>
       <c r="L275" s="4" t="n"/>
       <c r="M275" s="4" t="n"/>
-      <c r="N275" s="4" t="n"/>
     </row>
     <row r="276">
       <c r="A276" s="4" t="n"/>
@@ -5611,7 +5307,6 @@
       <c r="K276" s="4" t="n"/>
       <c r="L276" s="4" t="n"/>
       <c r="M276" s="4" t="n"/>
-      <c r="N276" s="4" t="n"/>
     </row>
     <row r="277">
       <c r="A277" s="4" t="n"/>
@@ -5627,7 +5322,6 @@
       <c r="K277" s="4" t="n"/>
       <c r="L277" s="4" t="n"/>
       <c r="M277" s="4" t="n"/>
-      <c r="N277" s="4" t="n"/>
     </row>
     <row r="278">
       <c r="A278" s="4" t="n"/>
@@ -5643,7 +5337,6 @@
       <c r="K278" s="4" t="n"/>
       <c r="L278" s="4" t="n"/>
       <c r="M278" s="4" t="n"/>
-      <c r="N278" s="4" t="n"/>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n"/>
@@ -5659,7 +5352,6 @@
       <c r="K279" s="4" t="n"/>
       <c r="L279" s="4" t="n"/>
       <c r="M279" s="4" t="n"/>
-      <c r="N279" s="4" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n"/>
@@ -5675,7 +5367,6 @@
       <c r="K280" s="4" t="n"/>
       <c r="L280" s="4" t="n"/>
       <c r="M280" s="4" t="n"/>
-      <c r="N280" s="4" t="n"/>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n"/>
@@ -5691,7 +5382,6 @@
       <c r="K281" s="4" t="n"/>
       <c r="L281" s="4" t="n"/>
       <c r="M281" s="4" t="n"/>
-      <c r="N281" s="4" t="n"/>
     </row>
     <row r="282">
       <c r="A282" s="4" t="n"/>
@@ -5707,7 +5397,6 @@
       <c r="K282" s="4" t="n"/>
       <c r="L282" s="4" t="n"/>
       <c r="M282" s="4" t="n"/>
-      <c r="N282" s="4" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n"/>
@@ -5723,7 +5412,6 @@
       <c r="K283" s="4" t="n"/>
       <c r="L283" s="4" t="n"/>
       <c r="M283" s="4" t="n"/>
-      <c r="N283" s="4" t="n"/>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n"/>
@@ -5739,7 +5427,6 @@
       <c r="K284" s="4" t="n"/>
       <c r="L284" s="4" t="n"/>
       <c r="M284" s="4" t="n"/>
-      <c r="N284" s="4" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n"/>
@@ -5755,7 +5442,6 @@
       <c r="K285" s="4" t="n"/>
       <c r="L285" s="4" t="n"/>
       <c r="M285" s="4" t="n"/>
-      <c r="N285" s="4" t="n"/>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n"/>
@@ -5771,7 +5457,6 @@
       <c r="K286" s="4" t="n"/>
       <c r="L286" s="4" t="n"/>
       <c r="M286" s="4" t="n"/>
-      <c r="N286" s="4" t="n"/>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n"/>
@@ -5787,7 +5472,6 @@
       <c r="K287" s="4" t="n"/>
       <c r="L287" s="4" t="n"/>
       <c r="M287" s="4" t="n"/>
-      <c r="N287" s="4" t="n"/>
     </row>
     <row r="288">
       <c r="A288" s="4" t="n"/>
@@ -5803,7 +5487,6 @@
       <c r="K288" s="4" t="n"/>
       <c r="L288" s="4" t="n"/>
       <c r="M288" s="4" t="n"/>
-      <c r="N288" s="4" t="n"/>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n"/>
@@ -5819,7 +5502,6 @@
       <c r="K289" s="4" t="n"/>
       <c r="L289" s="4" t="n"/>
       <c r="M289" s="4" t="n"/>
-      <c r="N289" s="4" t="n"/>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n"/>
@@ -5835,7 +5517,6 @@
       <c r="K290" s="4" t="n"/>
       <c r="L290" s="4" t="n"/>
       <c r="M290" s="4" t="n"/>
-      <c r="N290" s="4" t="n"/>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n"/>
@@ -5851,7 +5532,6 @@
       <c r="K291" s="4" t="n"/>
       <c r="L291" s="4" t="n"/>
       <c r="M291" s="4" t="n"/>
-      <c r="N291" s="4" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n"/>
@@ -5867,7 +5547,6 @@
       <c r="K292" s="4" t="n"/>
       <c r="L292" s="4" t="n"/>
       <c r="M292" s="4" t="n"/>
-      <c r="N292" s="4" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n"/>
@@ -5883,7 +5562,6 @@
       <c r="K293" s="4" t="n"/>
       <c r="L293" s="4" t="n"/>
       <c r="M293" s="4" t="n"/>
-      <c r="N293" s="4" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="4" t="n"/>
@@ -5899,7 +5577,6 @@
       <c r="K294" s="4" t="n"/>
       <c r="L294" s="4" t="n"/>
       <c r="M294" s="4" t="n"/>
-      <c r="N294" s="4" t="n"/>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n"/>
@@ -5915,7 +5592,6 @@
       <c r="K295" s="4" t="n"/>
       <c r="L295" s="4" t="n"/>
       <c r="M295" s="4" t="n"/>
-      <c r="N295" s="4" t="n"/>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n"/>
@@ -5931,7 +5607,6 @@
       <c r="K296" s="4" t="n"/>
       <c r="L296" s="4" t="n"/>
       <c r="M296" s="4" t="n"/>
-      <c r="N296" s="4" t="n"/>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n"/>
@@ -5947,7 +5622,6 @@
       <c r="K297" s="4" t="n"/>
       <c r="L297" s="4" t="n"/>
       <c r="M297" s="4" t="n"/>
-      <c r="N297" s="4" t="n"/>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n"/>
@@ -5963,7 +5637,6 @@
       <c r="K298" s="4" t="n"/>
       <c r="L298" s="4" t="n"/>
       <c r="M298" s="4" t="n"/>
-      <c r="N298" s="4" t="n"/>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n"/>
@@ -5979,7 +5652,6 @@
       <c r="K299" s="4" t="n"/>
       <c r="L299" s="4" t="n"/>
       <c r="M299" s="4" t="n"/>
-      <c r="N299" s="4" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n"/>
@@ -5995,7 +5667,6 @@
       <c r="K300" s="4" t="n"/>
       <c r="L300" s="4" t="n"/>
       <c r="M300" s="4" t="n"/>
-      <c r="N300" s="4" t="n"/>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n"/>
@@ -6011,7 +5682,6 @@
       <c r="K301" s="4" t="n"/>
       <c r="L301" s="4" t="n"/>
       <c r="M301" s="4" t="n"/>
-      <c r="N301" s="4" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n"/>
@@ -6027,7 +5697,6 @@
       <c r="K302" s="4" t="n"/>
       <c r="L302" s="4" t="n"/>
       <c r="M302" s="4" t="n"/>
-      <c r="N302" s="4" t="n"/>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n"/>
@@ -6043,7 +5712,6 @@
       <c r="K303" s="4" t="n"/>
       <c r="L303" s="4" t="n"/>
       <c r="M303" s="4" t="n"/>
-      <c r="N303" s="4" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="4" t="n"/>
@@ -6059,7 +5727,6 @@
       <c r="K304" s="4" t="n"/>
       <c r="L304" s="4" t="n"/>
       <c r="M304" s="4" t="n"/>
-      <c r="N304" s="4" t="n"/>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n"/>
@@ -6075,7 +5742,6 @@
       <c r="K305" s="4" t="n"/>
       <c r="L305" s="4" t="n"/>
       <c r="M305" s="4" t="n"/>
-      <c r="N305" s="4" t="n"/>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n"/>
@@ -6091,7 +5757,6 @@
       <c r="K306" s="4" t="n"/>
       <c r="L306" s="4" t="n"/>
       <c r="M306" s="4" t="n"/>
-      <c r="N306" s="4" t="n"/>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n"/>
@@ -6107,7 +5772,6 @@
       <c r="K307" s="4" t="n"/>
       <c r="L307" s="4" t="n"/>
       <c r="M307" s="4" t="n"/>
-      <c r="N307" s="4" t="n"/>
     </row>
     <row r="308">
       <c r="A308" s="4" t="n"/>
@@ -6123,7 +5787,6 @@
       <c r="K308" s="4" t="n"/>
       <c r="L308" s="4" t="n"/>
       <c r="M308" s="4" t="n"/>
-      <c r="N308" s="4" t="n"/>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n"/>
@@ -6139,7 +5802,6 @@
       <c r="K309" s="4" t="n"/>
       <c r="L309" s="4" t="n"/>
       <c r="M309" s="4" t="n"/>
-      <c r="N309" s="4" t="n"/>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n"/>
@@ -6155,7 +5817,6 @@
       <c r="K310" s="4" t="n"/>
       <c r="L310" s="4" t="n"/>
       <c r="M310" s="4" t="n"/>
-      <c r="N310" s="4" t="n"/>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n"/>
@@ -6171,7 +5832,6 @@
       <c r="K311" s="4" t="n"/>
       <c r="L311" s="4" t="n"/>
       <c r="M311" s="4" t="n"/>
-      <c r="N311" s="4" t="n"/>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n"/>
@@ -6187,7 +5847,6 @@
       <c r="K312" s="4" t="n"/>
       <c r="L312" s="4" t="n"/>
       <c r="M312" s="4" t="n"/>
-      <c r="N312" s="4" t="n"/>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n"/>
@@ -6203,7 +5862,6 @@
       <c r="K313" s="4" t="n"/>
       <c r="L313" s="4" t="n"/>
       <c r="M313" s="4" t="n"/>
-      <c r="N313" s="4" t="n"/>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n"/>
@@ -6219,7 +5877,6 @@
       <c r="K314" s="4" t="n"/>
       <c r="L314" s="4" t="n"/>
       <c r="M314" s="4" t="n"/>
-      <c r="N314" s="4" t="n"/>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n"/>
@@ -6235,7 +5892,6 @@
       <c r="K315" s="4" t="n"/>
       <c r="L315" s="4" t="n"/>
       <c r="M315" s="4" t="n"/>
-      <c r="N315" s="4" t="n"/>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n"/>
@@ -6251,7 +5907,6 @@
       <c r="K316" s="4" t="n"/>
       <c r="L316" s="4" t="n"/>
       <c r="M316" s="4" t="n"/>
-      <c r="N316" s="4" t="n"/>
     </row>
     <row r="317">
       <c r="A317" s="4" t="n"/>
@@ -6267,7 +5922,6 @@
       <c r="K317" s="4" t="n"/>
       <c r="L317" s="4" t="n"/>
       <c r="M317" s="4" t="n"/>
-      <c r="N317" s="4" t="n"/>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n"/>
@@ -6283,7 +5937,6 @@
       <c r="K318" s="4" t="n"/>
       <c r="L318" s="4" t="n"/>
       <c r="M318" s="4" t="n"/>
-      <c r="N318" s="4" t="n"/>
     </row>
     <row r="319">
       <c r="A319" s="4" t="n"/>
@@ -6299,7 +5952,6 @@
       <c r="K319" s="4" t="n"/>
       <c r="L319" s="4" t="n"/>
       <c r="M319" s="4" t="n"/>
-      <c r="N319" s="4" t="n"/>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n"/>
@@ -6315,7 +5967,6 @@
       <c r="K320" s="4" t="n"/>
       <c r="L320" s="4" t="n"/>
       <c r="M320" s="4" t="n"/>
-      <c r="N320" s="4" t="n"/>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n"/>
@@ -6331,7 +5982,6 @@
       <c r="K321" s="4" t="n"/>
       <c r="L321" s="4" t="n"/>
       <c r="M321" s="4" t="n"/>
-      <c r="N321" s="4" t="n"/>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n"/>
@@ -6347,7 +5997,6 @@
       <c r="K322" s="4" t="n"/>
       <c r="L322" s="4" t="n"/>
       <c r="M322" s="4" t="n"/>
-      <c r="N322" s="4" t="n"/>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n"/>
@@ -6363,7 +6012,6 @@
       <c r="K323" s="4" t="n"/>
       <c r="L323" s="4" t="n"/>
       <c r="M323" s="4" t="n"/>
-      <c r="N323" s="4" t="n"/>
     </row>
     <row r="324">
       <c r="A324" s="4" t="n"/>
@@ -6379,7 +6027,6 @@
       <c r="K324" s="4" t="n"/>
       <c r="L324" s="4" t="n"/>
       <c r="M324" s="4" t="n"/>
-      <c r="N324" s="4" t="n"/>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n"/>
@@ -6395,7 +6042,6 @@
       <c r="K325" s="4" t="n"/>
       <c r="L325" s="4" t="n"/>
       <c r="M325" s="4" t="n"/>
-      <c r="N325" s="4" t="n"/>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n"/>
@@ -6411,7 +6057,6 @@
       <c r="K326" s="4" t="n"/>
       <c r="L326" s="4" t="n"/>
       <c r="M326" s="4" t="n"/>
-      <c r="N326" s="4" t="n"/>
     </row>
     <row r="327">
       <c r="A327" s="4" t="n"/>
@@ -6427,7 +6072,6 @@
       <c r="K327" s="4" t="n"/>
       <c r="L327" s="4" t="n"/>
       <c r="M327" s="4" t="n"/>
-      <c r="N327" s="4" t="n"/>
     </row>
     <row r="328">
       <c r="A328" s="4" t="n"/>
@@ -6443,7 +6087,6 @@
       <c r="K328" s="4" t="n"/>
       <c r="L328" s="4" t="n"/>
       <c r="M328" s="4" t="n"/>
-      <c r="N328" s="4" t="n"/>
     </row>
     <row r="329">
       <c r="A329" s="4" t="n"/>
@@ -6459,7 +6102,6 @@
       <c r="K329" s="4" t="n"/>
       <c r="L329" s="4" t="n"/>
       <c r="M329" s="4" t="n"/>
-      <c r="N329" s="4" t="n"/>
     </row>
     <row r="330">
       <c r="A330" s="4" t="n"/>
@@ -6475,7 +6117,6 @@
       <c r="K330" s="4" t="n"/>
       <c r="L330" s="4" t="n"/>
       <c r="M330" s="4" t="n"/>
-      <c r="N330" s="4" t="n"/>
     </row>
     <row r="331">
       <c r="A331" s="4" t="n"/>
@@ -6491,7 +6132,6 @@
       <c r="K331" s="4" t="n"/>
       <c r="L331" s="4" t="n"/>
       <c r="M331" s="4" t="n"/>
-      <c r="N331" s="4" t="n"/>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n"/>
@@ -6507,7 +6147,6 @@
       <c r="K332" s="4" t="n"/>
       <c r="L332" s="4" t="n"/>
       <c r="M332" s="4" t="n"/>
-      <c r="N332" s="4" t="n"/>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n"/>
@@ -6523,7 +6162,6 @@
       <c r="K333" s="4" t="n"/>
       <c r="L333" s="4" t="n"/>
       <c r="M333" s="4" t="n"/>
-      <c r="N333" s="4" t="n"/>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n"/>
@@ -6539,7 +6177,6 @@
       <c r="K334" s="4" t="n"/>
       <c r="L334" s="4" t="n"/>
       <c r="M334" s="4" t="n"/>
-      <c r="N334" s="4" t="n"/>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n"/>
@@ -6555,7 +6192,6 @@
       <c r="K335" s="4" t="n"/>
       <c r="L335" s="4" t="n"/>
       <c r="M335" s="4" t="n"/>
-      <c r="N335" s="4" t="n"/>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n"/>
@@ -6571,7 +6207,6 @@
       <c r="K336" s="4" t="n"/>
       <c r="L336" s="4" t="n"/>
       <c r="M336" s="4" t="n"/>
-      <c r="N336" s="4" t="n"/>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n"/>
@@ -6587,7 +6222,6 @@
       <c r="K337" s="4" t="n"/>
       <c r="L337" s="4" t="n"/>
       <c r="M337" s="4" t="n"/>
-      <c r="N337" s="4" t="n"/>
     </row>
     <row r="338">
       <c r="A338" s="4" t="n"/>
@@ -6603,7 +6237,6 @@
       <c r="K338" s="4" t="n"/>
       <c r="L338" s="4" t="n"/>
       <c r="M338" s="4" t="n"/>
-      <c r="N338" s="4" t="n"/>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n"/>
@@ -6619,7 +6252,6 @@
       <c r="K339" s="4" t="n"/>
       <c r="L339" s="4" t="n"/>
       <c r="M339" s="4" t="n"/>
-      <c r="N339" s="4" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n"/>
@@ -6635,7 +6267,6 @@
       <c r="K340" s="4" t="n"/>
       <c r="L340" s="4" t="n"/>
       <c r="M340" s="4" t="n"/>
-      <c r="N340" s="4" t="n"/>
     </row>
     <row r="341">
       <c r="A341" s="4" t="n"/>
@@ -6651,7 +6282,6 @@
       <c r="K341" s="4" t="n"/>
       <c r="L341" s="4" t="n"/>
       <c r="M341" s="4" t="n"/>
-      <c r="N341" s="4" t="n"/>
     </row>
     <row r="342">
       <c r="A342" s="4" t="n"/>
@@ -6667,7 +6297,6 @@
       <c r="K342" s="4" t="n"/>
       <c r="L342" s="4" t="n"/>
       <c r="M342" s="4" t="n"/>
-      <c r="N342" s="4" t="n"/>
     </row>
     <row r="343">
       <c r="A343" s="4" t="n"/>
@@ -6683,7 +6312,6 @@
       <c r="K343" s="4" t="n"/>
       <c r="L343" s="4" t="n"/>
       <c r="M343" s="4" t="n"/>
-      <c r="N343" s="4" t="n"/>
     </row>
     <row r="344">
       <c r="A344" s="4" t="n"/>
@@ -6699,7 +6327,6 @@
       <c r="K344" s="4" t="n"/>
       <c r="L344" s="4" t="n"/>
       <c r="M344" s="4" t="n"/>
-      <c r="N344" s="4" t="n"/>
     </row>
     <row r="345">
       <c r="A345" s="4" t="n"/>
@@ -6715,7 +6342,6 @@
       <c r="K345" s="4" t="n"/>
       <c r="L345" s="4" t="n"/>
       <c r="M345" s="4" t="n"/>
-      <c r="N345" s="4" t="n"/>
     </row>
     <row r="346">
       <c r="A346" s="4" t="n"/>
@@ -6731,7 +6357,6 @@
       <c r="K346" s="4" t="n"/>
       <c r="L346" s="4" t="n"/>
       <c r="M346" s="4" t="n"/>
-      <c r="N346" s="4" t="n"/>
     </row>
     <row r="347">
       <c r="A347" s="4" t="n"/>
@@ -6747,7 +6372,6 @@
       <c r="K347" s="4" t="n"/>
       <c r="L347" s="4" t="n"/>
       <c r="M347" s="4" t="n"/>
-      <c r="N347" s="4" t="n"/>
     </row>
     <row r="348">
       <c r="A348" s="4" t="n"/>
@@ -6763,7 +6387,6 @@
       <c r="K348" s="4" t="n"/>
       <c r="L348" s="4" t="n"/>
       <c r="M348" s="4" t="n"/>
-      <c r="N348" s="4" t="n"/>
     </row>
     <row r="349">
       <c r="A349" s="4" t="n"/>
@@ -6779,7 +6402,6 @@
       <c r="K349" s="4" t="n"/>
       <c r="L349" s="4" t="n"/>
       <c r="M349" s="4" t="n"/>
-      <c r="N349" s="4" t="n"/>
     </row>
     <row r="350">
       <c r="A350" s="4" t="n"/>
@@ -6795,7 +6417,6 @@
       <c r="K350" s="4" t="n"/>
       <c r="L350" s="4" t="n"/>
       <c r="M350" s="4" t="n"/>
-      <c r="N350" s="4" t="n"/>
     </row>
     <row r="351">
       <c r="A351" s="4" t="n"/>
@@ -6811,7 +6432,6 @@
       <c r="K351" s="4" t="n"/>
       <c r="L351" s="4" t="n"/>
       <c r="M351" s="4" t="n"/>
-      <c r="N351" s="4" t="n"/>
     </row>
     <row r="352">
       <c r="A352" s="4" t="n"/>
@@ -6827,7 +6447,6 @@
       <c r="K352" s="4" t="n"/>
       <c r="L352" s="4" t="n"/>
       <c r="M352" s="4" t="n"/>
-      <c r="N352" s="4" t="n"/>
     </row>
     <row r="353">
       <c r="A353" s="4" t="n"/>
@@ -6843,7 +6462,6 @@
       <c r="K353" s="4" t="n"/>
       <c r="L353" s="4" t="n"/>
       <c r="M353" s="4" t="n"/>
-      <c r="N353" s="4" t="n"/>
     </row>
     <row r="354">
       <c r="A354" s="4" t="n"/>
@@ -6859,7 +6477,6 @@
       <c r="K354" s="4" t="n"/>
       <c r="L354" s="4" t="n"/>
       <c r="M354" s="4" t="n"/>
-      <c r="N354" s="4" t="n"/>
     </row>
     <row r="355">
       <c r="A355" s="4" t="n"/>
@@ -6875,7 +6492,6 @@
       <c r="K355" s="4" t="n"/>
       <c r="L355" s="4" t="n"/>
       <c r="M355" s="4" t="n"/>
-      <c r="N355" s="4" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="4" t="n"/>
@@ -6891,7 +6507,6 @@
       <c r="K356" s="4" t="n"/>
       <c r="L356" s="4" t="n"/>
       <c r="M356" s="4" t="n"/>
-      <c r="N356" s="4" t="n"/>
     </row>
     <row r="357">
       <c r="A357" s="4" t="n"/>
@@ -6907,7 +6522,6 @@
       <c r="K357" s="4" t="n"/>
       <c r="L357" s="4" t="n"/>
       <c r="M357" s="4" t="n"/>
-      <c r="N357" s="4" t="n"/>
     </row>
     <row r="358">
       <c r="A358" s="4" t="n"/>
@@ -6923,7 +6537,6 @@
       <c r="K358" s="4" t="n"/>
       <c r="L358" s="4" t="n"/>
       <c r="M358" s="4" t="n"/>
-      <c r="N358" s="4" t="n"/>
     </row>
     <row r="359">
       <c r="A359" s="4" t="n"/>
@@ -6939,7 +6552,6 @@
       <c r="K359" s="4" t="n"/>
       <c r="L359" s="4" t="n"/>
       <c r="M359" s="4" t="n"/>
-      <c r="N359" s="4" t="n"/>
     </row>
     <row r="360">
       <c r="A360" s="4" t="n"/>
@@ -6955,7 +6567,6 @@
       <c r="K360" s="4" t="n"/>
       <c r="L360" s="4" t="n"/>
       <c r="M360" s="4" t="n"/>
-      <c r="N360" s="4" t="n"/>
     </row>
     <row r="361">
       <c r="A361" s="4" t="n"/>
@@ -6971,7 +6582,6 @@
       <c r="K361" s="4" t="n"/>
       <c r="L361" s="4" t="n"/>
       <c r="M361" s="4" t="n"/>
-      <c r="N361" s="4" t="n"/>
     </row>
     <row r="362">
       <c r="A362" s="4" t="n"/>
@@ -6987,7 +6597,6 @@
       <c r="K362" s="4" t="n"/>
       <c r="L362" s="4" t="n"/>
       <c r="M362" s="4" t="n"/>
-      <c r="N362" s="4" t="n"/>
     </row>
     <row r="363">
       <c r="A363" s="4" t="n"/>
@@ -7003,7 +6612,6 @@
       <c r="K363" s="4" t="n"/>
       <c r="L363" s="4" t="n"/>
       <c r="M363" s="4" t="n"/>
-      <c r="N363" s="4" t="n"/>
     </row>
     <row r="364">
       <c r="A364" s="4" t="n"/>
@@ -7019,7 +6627,6 @@
       <c r="K364" s="4" t="n"/>
       <c r="L364" s="4" t="n"/>
       <c r="M364" s="4" t="n"/>
-      <c r="N364" s="4" t="n"/>
     </row>
     <row r="365">
       <c r="A365" s="4" t="n"/>
@@ -7035,7 +6642,6 @@
       <c r="K365" s="4" t="n"/>
       <c r="L365" s="4" t="n"/>
       <c r="M365" s="4" t="n"/>
-      <c r="N365" s="4" t="n"/>
     </row>
     <row r="366">
       <c r="A366" s="4" t="n"/>
@@ -7051,7 +6657,6 @@
       <c r="K366" s="4" t="n"/>
       <c r="L366" s="4" t="n"/>
       <c r="M366" s="4" t="n"/>
-      <c r="N366" s="4" t="n"/>
     </row>
     <row r="367">
       <c r="A367" s="4" t="n"/>
@@ -7067,7 +6672,6 @@
       <c r="K367" s="4" t="n"/>
       <c r="L367" s="4" t="n"/>
       <c r="M367" s="4" t="n"/>
-      <c r="N367" s="4" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="4" t="n"/>
@@ -7083,7 +6687,6 @@
       <c r="K368" s="4" t="n"/>
       <c r="L368" s="4" t="n"/>
       <c r="M368" s="4" t="n"/>
-      <c r="N368" s="4" t="n"/>
     </row>
     <row r="369">
       <c r="A369" s="4" t="n"/>
@@ -7099,7 +6702,6 @@
       <c r="K369" s="4" t="n"/>
       <c r="L369" s="4" t="n"/>
       <c r="M369" s="4" t="n"/>
-      <c r="N369" s="4" t="n"/>
     </row>
     <row r="370">
       <c r="A370" s="4" t="n"/>
@@ -7115,7 +6717,6 @@
       <c r="K370" s="4" t="n"/>
       <c r="L370" s="4" t="n"/>
       <c r="M370" s="4" t="n"/>
-      <c r="N370" s="4" t="n"/>
     </row>
     <row r="371">
       <c r="A371" s="4" t="n"/>
@@ -7131,7 +6732,6 @@
       <c r="K371" s="4" t="n"/>
       <c r="L371" s="4" t="n"/>
       <c r="M371" s="4" t="n"/>
-      <c r="N371" s="4" t="n"/>
     </row>
     <row r="372">
       <c r="A372" s="4" t="n"/>
@@ -7147,7 +6747,6 @@
       <c r="K372" s="4" t="n"/>
       <c r="L372" s="4" t="n"/>
       <c r="M372" s="4" t="n"/>
-      <c r="N372" s="4" t="n"/>
     </row>
     <row r="373">
       <c r="A373" s="4" t="n"/>
@@ -7163,7 +6762,6 @@
       <c r="K373" s="4" t="n"/>
       <c r="L373" s="4" t="n"/>
       <c r="M373" s="4" t="n"/>
-      <c r="N373" s="4" t="n"/>
     </row>
     <row r="374">
       <c r="A374" s="4" t="n"/>
@@ -7179,7 +6777,6 @@
       <c r="K374" s="4" t="n"/>
       <c r="L374" s="4" t="n"/>
       <c r="M374" s="4" t="n"/>
-      <c r="N374" s="4" t="n"/>
     </row>
     <row r="375">
       <c r="A375" s="4" t="n"/>
@@ -7195,7 +6792,6 @@
       <c r="K375" s="4" t="n"/>
       <c r="L375" s="4" t="n"/>
       <c r="M375" s="4" t="n"/>
-      <c r="N375" s="4" t="n"/>
     </row>
     <row r="376">
       <c r="A376" s="4" t="n"/>
@@ -7211,7 +6807,6 @@
       <c r="K376" s="4" t="n"/>
       <c r="L376" s="4" t="n"/>
       <c r="M376" s="4" t="n"/>
-      <c r="N376" s="4" t="n"/>
     </row>
     <row r="377">
       <c r="A377" s="4" t="n"/>
@@ -7227,7 +6822,6 @@
       <c r="K377" s="4" t="n"/>
       <c r="L377" s="4" t="n"/>
       <c r="M377" s="4" t="n"/>
-      <c r="N377" s="4" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="4" t="n"/>
@@ -7243,7 +6837,6 @@
       <c r="K378" s="4" t="n"/>
       <c r="L378" s="4" t="n"/>
       <c r="M378" s="4" t="n"/>
-      <c r="N378" s="4" t="n"/>
     </row>
     <row r="379">
       <c r="A379" s="4" t="n"/>
@@ -7259,7 +6852,6 @@
       <c r="K379" s="4" t="n"/>
       <c r="L379" s="4" t="n"/>
       <c r="M379" s="4" t="n"/>
-      <c r="N379" s="4" t="n"/>
     </row>
     <row r="380">
       <c r="A380" s="4" t="n"/>
@@ -7275,7 +6867,6 @@
       <c r="K380" s="4" t="n"/>
       <c r="L380" s="4" t="n"/>
       <c r="M380" s="4" t="n"/>
-      <c r="N380" s="4" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="4" t="n"/>
@@ -7291,7 +6882,6 @@
       <c r="K381" s="4" t="n"/>
       <c r="L381" s="4" t="n"/>
       <c r="M381" s="4" t="n"/>
-      <c r="N381" s="4" t="n"/>
     </row>
     <row r="382">
       <c r="A382" s="4" t="n"/>
@@ -7307,7 +6897,6 @@
       <c r="K382" s="4" t="n"/>
       <c r="L382" s="4" t="n"/>
       <c r="M382" s="4" t="n"/>
-      <c r="N382" s="4" t="n"/>
     </row>
     <row r="383">
       <c r="A383" s="4" t="n"/>
@@ -7323,7 +6912,6 @@
       <c r="K383" s="4" t="n"/>
       <c r="L383" s="4" t="n"/>
       <c r="M383" s="4" t="n"/>
-      <c r="N383" s="4" t="n"/>
     </row>
     <row r="384">
       <c r="A384" s="4" t="n"/>
@@ -7339,7 +6927,6 @@
       <c r="K384" s="4" t="n"/>
       <c r="L384" s="4" t="n"/>
       <c r="M384" s="4" t="n"/>
-      <c r="N384" s="4" t="n"/>
     </row>
     <row r="385">
       <c r="A385" s="4" t="n"/>
@@ -7355,7 +6942,6 @@
       <c r="K385" s="4" t="n"/>
       <c r="L385" s="4" t="n"/>
       <c r="M385" s="4" t="n"/>
-      <c r="N385" s="4" t="n"/>
     </row>
     <row r="386">
       <c r="A386" s="4" t="n"/>
@@ -7371,7 +6957,6 @@
       <c r="K386" s="4" t="n"/>
       <c r="L386" s="4" t="n"/>
       <c r="M386" s="4" t="n"/>
-      <c r="N386" s="4" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="4" t="n"/>
@@ -7387,7 +6972,6 @@
       <c r="K387" s="4" t="n"/>
       <c r="L387" s="4" t="n"/>
       <c r="M387" s="4" t="n"/>
-      <c r="N387" s="4" t="n"/>
     </row>
     <row r="388">
       <c r="A388" s="4" t="n"/>
@@ -7403,7 +6987,6 @@
       <c r="K388" s="4" t="n"/>
       <c r="L388" s="4" t="n"/>
       <c r="M388" s="4" t="n"/>
-      <c r="N388" s="4" t="n"/>
     </row>
     <row r="389">
       <c r="A389" s="4" t="n"/>
@@ -7419,7 +7002,6 @@
       <c r="K389" s="4" t="n"/>
       <c r="L389" s="4" t="n"/>
       <c r="M389" s="4" t="n"/>
-      <c r="N389" s="4" t="n"/>
     </row>
     <row r="390">
       <c r="A390" s="4" t="n"/>
@@ -7435,7 +7017,6 @@
       <c r="K390" s="4" t="n"/>
       <c r="L390" s="4" t="n"/>
       <c r="M390" s="4" t="n"/>
-      <c r="N390" s="4" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="4" t="n"/>
@@ -7451,7 +7032,6 @@
       <c r="K391" s="4" t="n"/>
       <c r="L391" s="4" t="n"/>
       <c r="M391" s="4" t="n"/>
-      <c r="N391" s="4" t="n"/>
     </row>
     <row r="392">
       <c r="A392" s="4" t="n"/>
@@ -7467,7 +7047,6 @@
       <c r="K392" s="4" t="n"/>
       <c r="L392" s="4" t="n"/>
       <c r="M392" s="4" t="n"/>
-      <c r="N392" s="4" t="n"/>
     </row>
     <row r="393">
       <c r="A393" s="4" t="n"/>
@@ -7483,7 +7062,6 @@
       <c r="K393" s="4" t="n"/>
       <c r="L393" s="4" t="n"/>
       <c r="M393" s="4" t="n"/>
-      <c r="N393" s="4" t="n"/>
     </row>
     <row r="394">
       <c r="A394" s="4" t="n"/>
@@ -7499,7 +7077,6 @@
       <c r="K394" s="4" t="n"/>
       <c r="L394" s="4" t="n"/>
       <c r="M394" s="4" t="n"/>
-      <c r="N394" s="4" t="n"/>
     </row>
     <row r="395">
       <c r="A395" s="4" t="n"/>
@@ -7515,7 +7092,6 @@
       <c r="K395" s="4" t="n"/>
       <c r="L395" s="4" t="n"/>
       <c r="M395" s="4" t="n"/>
-      <c r="N395" s="4" t="n"/>
     </row>
     <row r="396">
       <c r="A396" s="4" t="n"/>
@@ -7531,7 +7107,6 @@
       <c r="K396" s="4" t="n"/>
       <c r="L396" s="4" t="n"/>
       <c r="M396" s="4" t="n"/>
-      <c r="N396" s="4" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="4" t="n"/>
@@ -7547,7 +7122,6 @@
       <c r="K397" s="4" t="n"/>
       <c r="L397" s="4" t="n"/>
       <c r="M397" s="4" t="n"/>
-      <c r="N397" s="4" t="n"/>
     </row>
     <row r="398">
       <c r="A398" s="4" t="n"/>
@@ -7563,7 +7137,6 @@
       <c r="K398" s="4" t="n"/>
       <c r="L398" s="4" t="n"/>
       <c r="M398" s="4" t="n"/>
-      <c r="N398" s="4" t="n"/>
     </row>
     <row r="399">
       <c r="A399" s="4" t="n"/>
@@ -7579,7 +7152,6 @@
       <c r="K399" s="4" t="n"/>
       <c r="L399" s="4" t="n"/>
       <c r="M399" s="4" t="n"/>
-      <c r="N399" s="4" t="n"/>
     </row>
     <row r="400">
       <c r="A400" s="4" t="n"/>
@@ -7595,7 +7167,6 @@
       <c r="K400" s="4" t="n"/>
       <c r="L400" s="4" t="n"/>
       <c r="M400" s="4" t="n"/>
-      <c r="N400" s="4" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -21957,10 +21528,15 @@
           <t>email</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>jungyunlee@yuhs.ac
+GLORY.drylab@gmail.com</t>
+        </is>
+      </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>대표 이메일 (비워 두면 표시되지 않음)</t>
+          <t>이메일. 여러 개면 한 칸 안에서 Alt+Enter 로 줄을 바꿔 적습니다 (쉼표로 구분해도 됩니다). 비워 두면 표시되지 않음</t>
         </is>
       </c>
     </row>

</xml_diff>